<commit_message>
Update states, message and save/load
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -5940,7 +5941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
@@ -6070,12 +6071,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MENU_SAVE</t>
+          <t>MENU_SAVE_FILE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Save File</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -6087,119 +6088,153 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MENU_LOAD</t>
+          <t>MENU_EXIT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Load File</t>
+          <t>Exit Game</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>读档</t>
+          <t>回到标题</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MENU_EXIT</t>
+          <t>DIALOGUE_BOOK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Exit Game</t>
+          <t>Dialogue Book</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>回到标题</t>
+          <t>对话手册</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DIALOGUE_BOOK</t>
+          <t>DIALOGUE_BOOK_DESC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dialogue Book</t>
+          <t>You can review the dialogues that you've met with it.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>对话手册</t>
+          <t>持有后可以查看经历过的对话内容。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DIALOGUE_BOOK_DESC</t>
+          <t>EQUIP_UNEQUIPPED</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>You can review the dialogues that you've met with it.</t>
+          <t>[Unequipped]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>持有后可以查看经历过的对话内容。</t>
+          <t>[未装备]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>EQUIP_UNEQUIPPED</t>
+          <t>EQUIP_UNEQUIP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[Unequipped]</t>
+          <t>Unequip</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[未装备]</t>
+          <t>卸下</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EQUIP_UNEQUIP</t>
+          <t>EQUIP_UNEQUIP_DESC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Unequip</t>
+          <t>Remove equipment from this slot.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>卸下</t>
+          <t>卸下当前槽位的装备。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EQUIP_UNEQUIP_DESC</t>
+          <t>MENU_SAVE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Remove equipment from this slot.</t>
+          <t>Save File</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>卸下当前槽位的装备。</t>
+          <t>存档</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MENU_LOAD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Load File</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>读档</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MENU_LOAD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Load File</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>读档</t>
         </is>
       </c>
     </row>
@@ -6647,4 +6682,69 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>en_GB</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zh_CN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>POISONED</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Poisoned</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>中毒</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>POISONED_DESC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Once afflicted with the Poisoned status, the affected entity loses additional HP equal to the number of Poison stacks at the end of each turn.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>陷入中毒状态后每回合会多损失中毒层数数值的生命值</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update stairs and teleport
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C350"/>
+  <dimension ref="A1:C362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -6368,6 +6368,210 @@
       <c r="C350" t="inlineStr">
         <is>
           <t>通过 ID 从任意战斗者移除状态，并触发其 onRemove 蓝图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>OPEN_SHOP</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Open Shop</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>打开商店</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>OPEN_SHOP_DESC</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Open the map shop with purchasable item IDs and whether selling is allowed.</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>打开地图场景商店，参数为可购买道具ID数组和是否允许出售。</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>RECORD_TELEPOINT</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Record Telepoint</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>记录传送点</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>RECORD_TELEPOINT_DESC</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Record a telepoint for a map so it can be used by teleport items.</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>记录地图传送点，供传送道具使用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>OPEN_MONSTER_BOOK</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Open Monster Book</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>打开怪物手册</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>OPEN_MONSTER_BOOK_DESC</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Open the monster handbook for the current map.</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>打开当前地图的怪物手册。</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>GET_CURRENT_REGION</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Get Current Region</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>获取当前区域</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>GET_CURRENT_REGION_DESC</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Get the current mota region name.</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>获取当前魔塔区域名。</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>SET_CURRENT_REGION</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Set Current Region</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>设置当前区域</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>SET_CURRENT_REGION_DESC</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Set the current mota region name.</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>设置当前魔塔区域名。</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>OPEN_FLOOR_TELEPORTER</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Open Floor Teleporter</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>打开楼层传送器</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>OPEN_FLOOR_TELEPORTER_DESC</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Open the visited-floor teleporter preview window.</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>打开已去过楼层的传送器预览窗口。</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
@@ -6728,40 +6932,6 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>出售</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>OPEN_SHOP</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Open Shop</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>打开商店</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>OPEN_SHOP_DESC</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Open the map shop with purchasable item IDs and whether selling is allowed.</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>打开地图场景商店，参数为可购买道具ID数组和是否允许出售。</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.75" customWidth="1" min="1" max="1"/>
@@ -6934,6 +7104,40 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>持有后可以查看敌人信息（快捷键D）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FLY_FLOOR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Teleporter</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>地图传送器</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FLY_FLOOR_DESC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>You can teleport to the map you had been to with it(Hotkey: F).</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>持有后可以在前往过的传送点（快捷键F）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update consumables, maps and configs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -4014,15 +4015,13 @@
           <t>EQUALS</t>
         </is>
       </c>
-      <c r="B212" s="1" t="inlineStr">
-        <is>
-          <t>==</t>
-        </is>
-      </c>
-      <c r="C212" s="1" t="inlineStr">
-        <is>
-          <t>==</t>
-        </is>
+      <c r="B212" s="1">
+        <f>=</f>
+        <v/>
+      </c>
+      <c r="C212" s="1">
+        <f>=</f>
+        <v/>
       </c>
     </row>
     <row r="213">
@@ -6587,7 +6586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
@@ -6932,6 +6931,23 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>出售</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>POINT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>P {index}</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>点位 {index}</t>
         </is>
       </c>
     </row>
@@ -7478,4 +7494,69 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>en_GB</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zh_CN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MAP_01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tower G</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>魔塔 0 层</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MAP_02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tower 1F</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>魔塔 1 层</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update damage particle, items
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C362"/>
+  <dimension ref="A1:C372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -6571,6 +6571,176 @@
       <c r="C362" t="inlineStr">
         <is>
           <t>打开已去过楼层的传送器预览窗口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>DESTROY_TERRAIN</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Destroy Terrain</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>破坏地形</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>DESTROY_TERRAIN_DESC</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Replace one tile on a layer of the current map with the specified tile ID.</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>将当前地图指定图层上的一个格子替换为指定 tileID。</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>GET_TERRAIN_TILE</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Get Terrain Tile</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>获取地形 Tile</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>GET_TERRAIN_TILE_DESC</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Get the tile ID at a layer position on the current map.</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>获取当前地图指定图层和坐标上的 tileID。</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>GET_PLAYER_FRONT_POSITION</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Get Player Front Position</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>获取玩家面前坐标</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>GET_PLAYER_FRONT_POSITION_DESC</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Get the tile coordinate in front of the player based on the current facing direction.</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>根据玩家当前朝向获取面前一格的地图坐标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>DESTROY_TERRAIN_LIST</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Destroy Terrain List</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>批量破坏地形</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>DESTROY_TERRAIN_LIST_DESC</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Replace multiple tiles on a layer of the current map with the specified tile ID.</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>将当前地图指定图层上的多个格子替换为指定 tileID。</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>GET_TERRAIN_TILE_POSITIONS</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Get Terrain Tile Positions</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>获取地形 Tile 坐标列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>GET_TERRAIN_TILE_POSITIONS_DESC</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Get all coordinates matching a tile ID on a layer of the current map.</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>获取当前地图指定图层中所有匹配 tileID 的坐标。</t>
         </is>
       </c>
     </row>
@@ -6962,7 +7132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.75" customWidth="1" min="1" max="1"/>
@@ -7154,6 +7324,74 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>持有后可以在前往过的传送点（快捷键F）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BREAK_WALL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pickaxe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>镐</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BREAK_WALL_DESC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>You can use it to destroy a wall in front of you.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>可以破坏面前的一堵墙壁</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CLEAR_WALL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Earthquake Scroll</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>地震卷轴</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CLEAR_WALL_DESC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>You can use this to remove all walls on the current map.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>可以清除当前地图所有墙壁</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latent, animation, movement, light and rely meta
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C372"/>
+  <dimension ref="A1:C380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -6741,6 +6741,142 @@
       <c r="C372" t="inlineStr">
         <is>
           <t>获取当前地图指定图层中所有匹配 tileID 的坐标。</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>SET_MOVE_ROUTE</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Set Move Route</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>设置移动路线</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>SET_MOVE_ROUTE_DESC</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Set an actor movement route. Started continues immediately; Finished continues after movement ends.</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>设置 actor 的移动路线。Started 立即继续，Finished 在移动结束后继续。</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>SET_AUTO_PATH_TO_DESTINATION</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Set Auto Path to Destination</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>设置自动寻路到终点</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>SET_AUTO_PATH_TO_DESTINATION_DESC</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Pathfind an actor to the target map cell. Started continues immediately; Finished continues after movement ends.</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>让 actor 自动寻路到指定地图格。Started 立即继续，Finished 在移动结束后继续。</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>FREEZE_TRANSITION_BACKGROUND</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Freeze Transition Background</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>冻结转场背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>FREEZE_TRANSITION_BACKGROUND_DESC</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Capture the current frame as the next transition background, then continue when ready.</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>捕获当前帧作为下一次转场背景，并在捕获完成后继续。</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>REQUEST_TRANSITION</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Request Transition</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>请求转场</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>REQUEST_TRANSITION_DESC</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Start a screen transition (empty transitionName uses a plain fade), then continue when it finishes.</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>启动屏幕转场（transitionName 为空时为普通淡入），并在转场结束后继续。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update states, related bp, map, data and docs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C380"/>
+  <dimension ref="A1:C382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -6877,6 +6878,40 @@
       <c r="C380" t="inlineStr">
         <is>
           <t>启动屏幕转场（transitionName 为空时为普通淡入），并在转场结束后继续。</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>GAME_OVER</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Game Over</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>游戏结束</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>GAME_OVER_DESC</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Switch to the game over scene.</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>进入游戏结束场景。</t>
         </is>
       </c>
     </row>
@@ -7879,7 +7914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
@@ -7902,32 +7937,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POISONED</t>
+          <t>NORMAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Poisoned</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>中毒</t>
+          <t>正常</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>POISONED</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Poisoned</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>中毒</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>POISONED_DESC</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Once afflicted with the Poisoned status, the affected entity loses additional HP equal to the number of Poison stacks at the end of each turn.</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>陷入中毒状态后每回合会多损失中毒层数数值的生命值</t>
         </is>
@@ -8001,4 +8053,69 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>en_GB</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zh_CN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S_POISOING</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Poisoning</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>中毒</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S_POISOING_DESC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Player will be poisoned after this battle.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>战斗后会使我方陷入中毒状态</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update enemies and file selector
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -7392,7 +7392,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>可以打开一扇黄门</t>
+          <t>可以打开一扇黄门。</t>
         </is>
       </c>
     </row>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>可以打开一扇蓝门</t>
+          <t>可以打开一扇蓝门。</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>可以打开一扇红门</t>
+          <t>可以打开一扇红门。</t>
         </is>
       </c>
     </row>
@@ -7494,7 +7494,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>持有后可以查看敌人信息（快捷键D）</t>
+          <t>持有后可以查看敌人信息（快捷键D）。</t>
         </is>
       </c>
     </row>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>持有后可以在前往过的传送点（快捷键F）</t>
+          <t>持有后可以在前往过的传送点（快捷键F）。</t>
         </is>
       </c>
     </row>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>可以破坏面前的一堵墙壁</t>
+          <t>可以破坏面前的一堵墙壁。</t>
         </is>
       </c>
     </row>
@@ -7596,7 +7596,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>可以清除当前地图所有墙壁</t>
+          <t>可以清除当前地图所有墙壁。</t>
         </is>
       </c>
     </row>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>可以破坏面前的一块熔岩</t>
+          <t>可以破坏面前的一块熔岩。</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>可以破坏面前的一块冰墙</t>
+          <t>可以破坏面前的一块冰墙。</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>这是一个骷髅</t>
+          <t>这是一个骷髅。</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>这是一个史莱姆</t>
+          <t>这是一个史莱姆。</t>
         </is>
       </c>
     </row>
@@ -7834,7 +7834,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>铁制造的剑，装备后可提升10攻击力</t>
+          <t>铁制造的剑，装备后可提升10攻击力。</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>铁制造的盾，装备后可提升10防御力</t>
+          <t>铁制造的盾，装备后可提升10防御力。</t>
         </is>
       </c>
     </row>
@@ -7933,7 +7933,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>勇猛的战士，具有比较均衡的能力</t>
+          <t>勇猛的战士，具有比较均衡的能力。</t>
         </is>
       </c>
     </row>
@@ -7948,7 +7948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
@@ -8015,7 +8015,41 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>陷入中毒状态后每回合会多损失中毒层数数值的生命值</t>
+          <t>陷入中毒状态后，每回合会多损失中毒层数数值的生命值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WEAK</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>衰弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WEAK_DESC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>When weakened, the attack and defense capabilities will be reduced based on the corresponding stack value during combat.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>陷入衰弱状态后，会在战斗时少发挥响应层数数值的攻击力和防御力。</t>
         </is>
       </c>
     </row>
@@ -8095,7 +8129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8145,7 +8179,41 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>战斗后会使我方陷入中毒状态</t>
+          <t>战斗后会使我方陷入中毒状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S_WEAKEN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Weaken</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>衰弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S_WEAKEN_DESC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Player will be weak after this battle.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>战斗后会使我方陷入衰弱状态。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update docs, style and nodefunctions
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C384"/>
+  <dimension ref="A1:C388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -6946,6 +6946,74 @@
       <c r="C384" t="inlineStr">
         <is>
           <t>进入游戏结束场景。</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>LOCK_CAMERA</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Lock Camera</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>锁定镜头</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>LOCK_CAMERA_DESC</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Lock the current map camera to the player.</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>将当前地图镜头锁定到玩家身上。</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>UNLOCK_CAMERA</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Unlock Camera</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>解除镜头锁定</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>UNLOCK_CAMERA_DESC</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Stop the current map camera from following the player.</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>停止当前地图镜头跟随玩家。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update docs, UI and Engine part
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -416,7 +416,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C388"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
     <col width="61.83203125" customWidth="1" min="2" max="2"/>
@@ -7030,7 +7030,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -7406,7 +7406,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="25.75" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
@@ -7749,7 +7749,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="29.58203125" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
@@ -8333,7 +8333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8356,202 +8356,236 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S_POISOING</t>
+          <t>NORMAL_SPECIAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Poisoning</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>中毒</t>
+          <t>普通</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S_POISOING_DESC</t>
+          <t>MORE_SPECIAL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Player will be poisoned after this battle.</t>
+          <t>More...</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>战斗后会使我方陷入中毒状态。</t>
+          <t>更多...</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S_WEAKEN</t>
+          <t>S_POISONING</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Weaken</t>
+          <t>Poisoning</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>衰弱</t>
+          <t>中毒</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S_WEAKEN_DESC</t>
+          <t>S_POISONING_DESC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Player will be weak after this battle.</t>
+          <t>Player will be poisoned after this battle.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>战斗后会使我方陷入衰弱状态。</t>
+          <t>战斗后会使我方陷入中毒状态。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S_HARD</t>
+          <t>S_WEAKEN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Weaken</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>坚固</t>
+          <t>衰弱</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S_HARD_DESC</t>
+          <t>S_WEAKEN_DESC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The holder's DEF is treated as at least the opponent's ATK minus 1 during damage calculation.</t>
+          <t>Player will be weak after this battle.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>计算伤害时，持有者的防御力视为不低于对方攻击力-1。</t>
+          <t>战斗后会使我方陷入衰弱状态。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S_MAGIC</t>
+          <t>S_HARD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Magic</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>魔攻</t>
+          <t>坚固</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S_MAGIC_DESC</t>
+          <t>S_HARD_DESC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>During battle, the holder treats the opponent's DEF as 0 when calculating damage.</t>
+          <t>The holder's DEF is treated as at least the opponent's ATK minus 1 during damage calculation.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>战斗中计算伤害时，持有者将对方防御力视为0。</t>
+          <t>计算伤害时，持有者的防御力视为不低于对方攻击力-1。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S_MULTIHIT</t>
+          <t>S_MAGIC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MultiHit</t>
+          <t>Magic</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>连击</t>
+          <t>魔攻</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S_MULTIHIT_DESC</t>
+          <t>S_MAGIC_DESC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>During battle, each round's base damage is multiplied by the holder's hit count. Missing or invalid values count as 1, with a minimum of 1.</t>
+          <t>During battle, the holder treats the opponent's DEF as 0 when calculating damage.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>战斗中，持有者每回合基础伤害会按连击数倍计算。未设置或无效值视为1，最低为1。</t>
+          <t>战斗中计算伤害时，持有者将对方防御力视为0。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S_COMPETE</t>
+          <t>S_MULTIHIT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Compete</t>
+          <t>MultiHit</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>争斗</t>
+          <t>连击</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>S_MULTIHIT_DESC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>During battle, each round's base damage is multiplied by the holder's hit count. Missing or invalid values count as 1, with a minimum of 1.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>战斗中，持有者每回合基础伤害会按连击数倍计算。未设置或无效值视为1，最低为1。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>S_COMPETE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Compete</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>争斗</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>S_COMPETE_DESC</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>The holder's ATK is treated as at least the opponent's ATK.</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>持有者的攻击力视为不低于对方攻击力。</t>
         </is>

</xml_diff>

<commit_message>
Update docs, editor, file explorer, animation preview and obj samples
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -415,8 +415,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C388"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
+  <dimension ref="A1:C402"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
     <col width="61.83203125" customWidth="1" min="2" max="2"/>
@@ -4050,13 +4050,15 @@
           <t>EQUALS</t>
         </is>
       </c>
-      <c r="B214" s="1">
-        <f>=</f>
-        <v/>
-      </c>
-      <c r="C214" s="1">
-        <f>=</f>
-        <v/>
+      <c r="B214" s="1" t="inlineStr">
+        <is>
+          <t>==</t>
+        </is>
+      </c>
+      <c r="C214" s="1" t="inlineStr">
+        <is>
+          <t>==</t>
+        </is>
       </c>
     </row>
     <row r="215">
@@ -7014,6 +7016,244 @@
       <c r="C388" t="inlineStr">
         <is>
           <t>停止当前地图镜头跟随玩家。</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>REGISTER_EVENT_BUS</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Register EventBus</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>注册 EventBus</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>REGISTER_EVENT_BUS_DESC</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Subscribe an object event or method to an EventBus key.</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>将对象的事件或方法注册到 EventBus key。</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>TRIGGER_EVENT_BUS</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Trigger EventBus</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>触发 EventBus</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>TRIGGER_EVENT_BUS_DESC</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Post kwargs to an EventBus key; registered object events run on a later logic frame.</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>向指定 EventBus key 发送参数，已注册的对象事件会在后续逻辑帧执行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>REGISTER_EVENT_BUS_EVENT</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Register EventBus Event</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>注册 EventBus 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>REGISTER_EVENT_BUS_EVENT_DESC</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Subscribe an object blueprint event to an EventBus key. Event payload is ignored.</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>将对象的蓝图事件注册到 EventBus key，忽略事件参数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>TRIGGER_BLUEPRINT_EVENT</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Trigger Blueprint Event</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>触发蓝图事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>TRIGGER_BLUEPRINT_EVENT_DESC</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Trigger a blueprint event on an object without arguments.</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>不带参数地触发对象上的蓝图事件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>GET_GAME_VARIABLE_REF</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Get Game Variable Ref</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>获取游戏变量引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>GET_GAME_VARIABLE_REF_DESC</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Get a readable/writable reference to a game variable.</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>获取一个可读写的游戏变量引用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>UNREGISTER_EVENT_BUS</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Unregister EventBus</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>取消 EventBus 注册</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>UNREGISTER_EVENT_BUS_DESC</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Unsubscribe an object event or method from an EventBus key.</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>取消对象事件或方法对 EventBus key 的注册。</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>UNREGISTER_EVENT_BUS_EVENT</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Unregister EventBus Event</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>取消 EventBus 蓝图事件注册</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>UNREGISTER_EVENT_BUS_EVENT_DESC</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Unsubscribe an object blueprint event from an EventBus key.</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>取消对象蓝图事件对 EventBus key 的注册。</t>
         </is>
       </c>
     </row>
@@ -7029,8 +7269,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -7391,6 +7631,210 @@
       <c r="C21" t="inlineStr">
         <is>
           <t>点位 {index}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>语言</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>缩放</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>framerate</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Frame Rate</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>帧率</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>verticalsync</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Vertical Sync</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>垂直同步</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>musicon</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Music</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>音乐</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>musicvolume</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Music Volume</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>音乐音量</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>soundon</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Sound</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>音效</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>soundvolume</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Sound Volume</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>音效音量</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>voiceon</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>语音</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>voicevolume</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Voice Volume</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>语音音量</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>en_GB</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>zh_CN</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Simplified Chinese</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>简体中文</t>
         </is>
       </c>
     </row>
@@ -7406,7 +7850,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.75" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
@@ -7749,7 +8193,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="29.58203125" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Update animation, UI and events
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -15,6 +15,7 @@
     <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Player" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C402"/>
+  <dimension ref="A1:C404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -4050,15 +4051,13 @@
           <t>EQUALS</t>
         </is>
       </c>
-      <c r="B214" s="1" t="inlineStr">
-        <is>
-          <t>==</t>
-        </is>
-      </c>
-      <c r="C214" s="1" t="inlineStr">
-        <is>
-          <t>==</t>
-        </is>
+      <c r="B214" s="1">
+        <f>=</f>
+        <v/>
+      </c>
+      <c r="C214" s="1">
+        <f>=</f>
+        <v/>
       </c>
     </row>
     <row r="215">
@@ -7254,12 +7253,111 @@
       <c r="C402" t="inlineStr">
         <is>
           <t>取消对象蓝图事件对 EventBus key 的注册。</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>GET_ANIM_VISUAL_LENGTH</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Get Animation Visual Length</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>获取动画视觉时长</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>GET_ANIM_VISUAL_LENGTH_DESC</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Get the visual duration of an animation, excluding sound track length (seconds).</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>获取指定动画的视觉时长（秒），不包含音轨长度。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>en_GB</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zh_CN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BRAVOR</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bravor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>勇士</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BRAVOR_DESC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>This is a bravor player pawn.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>这是一个勇士形式角色。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -7269,7 +7367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
@@ -7835,6 +7933,159 @@
       <c r="C33" t="inlineStr">
         <is>
           <t>简体中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>STAT_HP</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HP:</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>生命:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>STAT_MAXHP</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MAXHP:</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>最大生命:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>STAT_ATK</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ATK:</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>攻击:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>STAT_DEF</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DEF:</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>防御:</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>STAT_EXP</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EXP:</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>经验:</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>STAT_GOLD</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>GOLD:</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>金币:</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>STAT_DMG</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DMG:</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>伤害:</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>STAT_HIT</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HIT:</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>连击:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>STAT_CRIT</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CRIT:</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>临界:</t>
         </is>
       </c>
     </row>
@@ -8992,12 +9243,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>During battle, each round's base damage is multiplied by the holder's hit count. Missing or invalid values count as 1, with a minimum of 1.</t>
+          <t>During battle, each round's base damage is multiplied by the holder's hit count.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>战斗中，持有者每回合基础伤害会按连击数倍计算。未设置或无效值视为1，最低为1。</t>
+          <t>战斗中，持有者每回合基础伤害会按连击数倍计算。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update UI, Input and editor
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Player" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C404"/>
+  <dimension ref="A1:C406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -7287,6 +7287,40 @@
       <c r="C404" t="inlineStr">
         <is>
           <t>获取指定动画的视觉时长（秒），不包含音轨长度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>TO_SHORT_NUMBER</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Short Number</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>数值缩写</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>TO_SHORT_NUMBER_DESC</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Shorten large numbers with k/m/b suffixes.</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>将较大的数字显示为 k/m/b 缩写。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update spatial sound, docs, bp editor and UI
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C406"/>
+  <dimension ref="A1:C412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -7321,6 +7321,108 @@
       <c r="C406" t="inlineStr">
         <is>
           <t>将较大的数字显示为 k/m/b 缩写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>SHOW_VOICE_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Show Voice Message</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>语音对话</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>SHOW_VOICE_MESSAGE_DESC</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Play a voice clip and show dialogue on the current map scene. refActorTag controls dialogue-window placement; refActor controls spatial voice position.</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>在当前地图场景中播放语音并显示对话。refActorTag 控制对话窗口位置；refActor 控制空间语音位置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>SHOW_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Show Message</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>显示对话</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>SHOW_MESSAGE_DESC</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Show dialogue on the current map scene. refActorTag controls dialogue-window placement.</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>在当前地图场景中显示对话。refActorTag 用于控制对话窗口位置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>SHOW_SELECTION</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Show Selection</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>显示选项</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>SHOW_SELECTION_DESC</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Show a selection window on the current map scene. refActorTag controls selection-window placement.</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>在当前地图场景中显示选项窗口。refActorTag 用于控制选项窗口位置。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate some python type to C++
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="280" yWindow="4710" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-35050" yWindow="4360" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Player" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -69,10 +69,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -416,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C412"/>
+  <dimension ref="A1:C420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -4051,13 +4052,15 @@
           <t>EQUALS</t>
         </is>
       </c>
-      <c r="B214" s="1">
-        <f>=</f>
-        <v/>
-      </c>
-      <c r="C214" s="1">
-        <f>=</f>
-        <v/>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>==</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>==</t>
+        </is>
       </c>
     </row>
     <row r="215">
@@ -7423,6 +7426,142 @@
       <c r="C412" t="inlineStr">
         <is>
           <t>在当前地图场景中显示选项窗口。refActorTag 用于控制选项窗口位置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>GET_PLAYER_ATTR_REF</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Get Player Attribute Ref</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>获取玩家属性引用</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>GET_PLAYER_ATTR_REF_DESC</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Get a readable/writable reference to a player attribute (e.g. HP, ATK, DEF, GOLD).</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>获取玩家指定属性的可读写引用（如 HP/ATK/DEF/GOLD）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>ADD_HP</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Add HP</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>增加HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>ADD_HP_DESC</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Add HP to the player (can be negative to subtract).</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>为玩家增加（或减少）HP。</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>ADD_ATK</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Add ATK</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>增加攻击力</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>ADD_ATK_DESC</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Add ATK to the player (can be negative to subtract).</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>为玩家增加（或减少）攻击力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>ADD_DEF</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Add DEF</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>增加防御力</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>ADD_DEF_DESC</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Add DEF to the player (can be negative to subtract).</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>为玩家增加（或减少）防御力。</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7578,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9100,7 +9239,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -9165,7 +9304,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Update tone, stairs, blocking and docs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C420"/>
+  <dimension ref="A1:C437"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -4054,12 +4054,12 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>==</t>
+          <t>'==</t>
         </is>
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>==</t>
+          <t>'==</t>
         </is>
       </c>
     </row>
@@ -7562,6 +7562,295 @@
       <c r="C420" t="inlineStr">
         <is>
           <t>为玩家增加（或减少）防御力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>TONE_SHADER_LOAD_FAILED</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Failed to load screen tone shader</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>画面色调着色器加载失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>CHANGE_SCREEN_TONE</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Change Screen Tone</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>更改画面色调</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>CHANGE_SCREEN_TONE_DESC</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Change the screen tone over time. Red, green, and blue range from -255 to 255; gray ranges from 0 to 255; duration is in seconds.</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>在指定时间内更改画面色调。红、绿、蓝范围为 -255 到 255；灰度范围为 0 到 255；持续时间单位为秒。</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>CLEAR_SCREEN_TONE</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Clear Screen Tone</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>清除画面色调</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>CLEAR_SCREEN_TONE_DESC</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Fade the screen tone back to normal over the given duration in seconds.</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>在指定秒数内将画面色调恢复为正常。</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>CREATE_ACTOR_FROM_BP_PATH</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Create Actor From BP Path</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>从蓝图路径创建 Actor</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>CREATE_ACTOR_FROM_BP_PATH_DESC</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Create an actor from a blueprint class path and spawn it on the current map.</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>根据蓝图类路径创建 Actor，并生成到当前地图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>ADD_TIMER</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Add Timer</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>添加计时器</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>ADD_TIMER_DESC</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Wait for a scene timer. If blocking is enabled, player movement and scene hotkeys are disabled until TimeUp.</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>等待场景计时器。如果启用阻塞，TimeUp 前玩家移动和场景快捷键不可用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>RECORD_DESTROYED_ACTOR</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Record Destroyed Actor</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>记录已销毁 Actor</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>RECORD_DESTROYED_ACTOR_DESC</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Record a destroyed actor for persistence on the current map scene.</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>在当前地图场景中记录一个已销毁 Actor，用于存档持久化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>SELF_RECORD_DESTROYED</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Self Record Destroyed</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>自身记录已销毁</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>SELF_RECORD_DESTROYED_DESC</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Record the blueprint owner as a destroyed actor for persistence on the current map scene.</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>将蓝图所有者记录为已销毁 Actor，用于在当前地图场景中持久化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>RECORD_AND_DESTROY_ACTOR</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Record And Destroy Actor</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>记录并销毁 Actor</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>RECORD_AND_DESTROY_ACTOR_DESC</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Record a destroyed actor for persistence and destroy it on the current map scene.</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>在当前地图场景中记录一个已销毁 Actor 并销毁它。</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>SELF_RECORD_AND_DESTROY</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Self Record And Destroy</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>自身记录并销毁</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>SELF_RECORD_AND_DESTROY_DESC</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Record the blueprint owner as destroyed for persistence and destroy it on the current map scene.</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>将蓝图所有者记录为已销毁并销毁它，用于在当前地图场景中持久化。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update advanced node functions
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C437"/>
+  <dimension ref="A1:C453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -7352,12 +7352,12 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Play a voice clip and show dialogue on the current map scene. refActorTag controls dialogue-window placement; refActor controls spatial voice position.</t>
+          <t>Play a non-spatial voice clip and show a dialogue message on the current map scene. refActorTag controls dialogue-window placement.</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>在当前地图场景中播放语音并显示对话。refActorTag 控制对话窗口位置；refActor 控制空间语音位置。</t>
+          <t>在当前地图场景中播放非空间语音并显示对话。refActorTag 控制对话窗口位置。</t>
         </is>
       </c>
     </row>
@@ -7851,6 +7851,278 @@
       <c r="C437" t="inlineStr">
         <is>
           <t>将蓝图所有者记录为已销毁并销毁它，用于在当前地图场景中持久化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>SHOW_REF_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Show Ref Message</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>显示引用消息</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>SHOW_REF_MESSAGE_DESC</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Show a dialogue message on the current map scene. Uses a direct actor reference for window placement.</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>在当前地图场景中显示对话，通过直接 Actor 引用进行窗口定位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>SHOW_VOICE_REF_MESSAGE</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Show Voice Ref Message</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>显示引用语音消息</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>SHOW_VOICE_REF_MESSAGE_DESC</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Play a spatial voice clip and show a dialogue message on the current map scene. Uses a direct actor reference for voice positioning.</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>在当前地图场景中播放空间语音并显示对话。通过直接 Actor 引用进行语音定位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>GET_SELF_ATTR</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Get Self Attr</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>获取自身属性</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>GET_SELF_ATTR_DESC</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Read an attribute value from the blueprint owner</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>读取蓝图拥有者的属性值</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>SET_SELF_ATTR</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Set Self Attr</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>设置自身属性</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>SET_SELF_ATTR_DESC</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Set an attribute value on the blueprint owner</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>设置蓝图拥有者的属性值</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>IF_PLAYER_OVERLAPS</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>If Player Overlaps</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>玩家是否重叠</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>IF_PLAYER_OVERLAPS_DESC</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Check if the player shares the same cell as the blueprint owner</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>判断玩家是否与蓝图拥有者处于同一格子</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>IF_GAME_VAR</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>If Game Var</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>判断游戏变量</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>IF_GAME_VAR_DESC</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Compare a game variable with a given value, returning a true/false branch</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>将游戏变量与给定值进行比较，返回真假分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>GET_ACTOR_BY_TAG</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Get Actor By Tag</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>按标签查找角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>GET_ACTOR_BY_TAG_DESC</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Find an actor by tag on the current map</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>在当前地图上按标签查找角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>GET_ALL_ACTORS</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Get All Actors</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>获取全部角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>GET_ALL_ACTORS_DESC</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Get a list of all actors on the current map</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>获取当前地图上的所有角色列表</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update assets, default bps, editor functions and docs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-35050" yWindow="4360" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Player" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C453"/>
+  <dimension ref="A1:C465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -7024,1105 +7024,1309 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>REGISTER_EVENT_BUS</t>
+          <t>ATTACH_CAMERA</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Register EventBus</t>
+          <t>Attach Camera</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>注册 EventBus</t>
+          <t>附着镜头</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>REGISTER_EVENT_BUS_DESC</t>
+          <t>ATTACH_CAMERA_DESC</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Subscribe an object event or method to an EventBus key.</t>
+          <t>Attach the current map camera to the specified actor. Pass None to detach and stop following.</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>将对象的事件或方法注册到 EventBus key。</t>
+          <t>将当前地图镜头附着到指定 Actor；传入 None 可取消附着并停止跟随。</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>TRIGGER_EVENT_BUS</t>
+          <t>MOVE_CAMERA</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Trigger EventBus</t>
+          <t>Move Camera</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>触发 EventBus</t>
+          <t>移动镜头</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>TRIGGER_EVENT_BUS_DESC</t>
+          <t>MOVE_CAMERA_DESC</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Post kwargs to an EventBus key; registered object events run on a later logic frame.</t>
+          <t>Move the current map camera by the given viewport offset and clamp it to the map bounds.</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>向指定 EventBus key 发送参数，已注册的对象事件会在后续逻辑帧执行。</t>
+          <t>按给定视口偏移移动当前地图镜头，并将结果自动钳制到地图范围内。</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>REGISTER_EVENT_BUS_EVENT</t>
+          <t>REGISTER_EVENT_BUS</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Register EventBus Event</t>
+          <t>Register EventBus</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>注册 EventBus 事件</t>
+          <t>注册 EventBus</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>REGISTER_EVENT_BUS_EVENT_DESC</t>
+          <t>REGISTER_EVENT_BUS_DESC</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Subscribe an object blueprint event to an EventBus key. Event payload is ignored.</t>
+          <t>Subscribe an object event or method to an EventBus key.</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>将对象的蓝图事件注册到 EventBus key，忽略事件参数。</t>
+          <t>将对象的事件或方法注册到 EventBus key。</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>TRIGGER_BLUEPRINT_EVENT</t>
+          <t>TRIGGER_EVENT_BUS</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Trigger Blueprint Event</t>
+          <t>Trigger EventBus</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>触发蓝图事件</t>
+          <t>触发 EventBus</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>TRIGGER_BLUEPRINT_EVENT_DESC</t>
+          <t>TRIGGER_EVENT_BUS_DESC</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Trigger a blueprint event on an object without arguments.</t>
+          <t>Post kwargs to an EventBus key; registered object events run on a later logic frame.</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>不带参数地触发对象上的蓝图事件。</t>
+          <t>向指定 EventBus key 发送参数，已注册的对象事件会在后续逻辑帧执行。</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>GET_GAME_VARIABLE_REF</t>
+          <t>REGISTER_EVENT_BUS_EVENT</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Get Game Variable Ref</t>
+          <t>Register EventBus Event</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>获取游戏变量引用</t>
+          <t>注册 EventBus 事件</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>GET_GAME_VARIABLE_REF_DESC</t>
+          <t>REGISTER_EVENT_BUS_EVENT_DESC</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Get a readable/writable reference to a game variable.</t>
+          <t>Subscribe an object blueprint event to an EventBus key. Event payload is ignored.</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>获取一个可读写的游戏变量引用。</t>
+          <t>将对象的蓝图事件注册到 EventBus key，忽略事件参数。</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>UNREGISTER_EVENT_BUS</t>
+          <t>TRIGGER_BLUEPRINT_EVENT</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Unregister EventBus</t>
+          <t>Trigger Blueprint Event</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>取消 EventBus 注册</t>
+          <t>触发蓝图事件</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>UNREGISTER_EVENT_BUS_DESC</t>
+          <t>TRIGGER_BLUEPRINT_EVENT_DESC</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Unsubscribe an object event or method from an EventBus key.</t>
+          <t>Trigger a blueprint event on an object without arguments.</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>取消对象事件或方法对 EventBus key 的注册。</t>
+          <t>不带参数地触发对象上的蓝图事件。</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>UNREGISTER_EVENT_BUS_EVENT</t>
+          <t>GET_GAME_VARIABLE_REF</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Unregister EventBus Event</t>
+          <t>Get Game Variable Ref</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>取消 EventBus 蓝图事件注册</t>
+          <t>获取游戏变量引用</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>UNREGISTER_EVENT_BUS_EVENT_DESC</t>
+          <t>GET_GAME_VARIABLE_REF_DESC</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Unsubscribe an object blueprint event from an EventBus key.</t>
+          <t>Get a readable/writable reference to a game variable.</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>取消对象蓝图事件对 EventBus key 的注册。</t>
+          <t>获取一个可读写的游戏变量引用。</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>GET_ANIM_VISUAL_LENGTH</t>
+          <t>UNREGISTER_EVENT_BUS</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Get Animation Visual Length</t>
+          <t>Unregister EventBus</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>获取动画视觉时长</t>
+          <t>取消 EventBus 注册</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>GET_ANIM_VISUAL_LENGTH_DESC</t>
+          <t>UNREGISTER_EVENT_BUS_DESC</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Get the visual duration of an animation, excluding sound track length (seconds).</t>
+          <t>Unsubscribe an object event or method from an EventBus key.</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>获取指定动画的视觉时长（秒），不包含音轨长度。</t>
+          <t>取消对象事件或方法对 EventBus key 的注册。</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>TO_SHORT_NUMBER</t>
+          <t>UNREGISTER_EVENT_BUS_EVENT</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Short Number</t>
+          <t>Unregister EventBus Event</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>数值缩写</t>
+          <t>取消 EventBus 蓝图事件注册</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>TO_SHORT_NUMBER_DESC</t>
+          <t>UNREGISTER_EVENT_BUS_EVENT_DESC</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Shorten large numbers with k/m/b suffixes.</t>
+          <t>Unsubscribe an object blueprint event from an EventBus key.</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>将较大的数字显示为 k/m/b 缩写。</t>
+          <t>取消对象蓝图事件对 EventBus key 的注册。</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>SHOW_VOICE_MESSAGE</t>
+          <t>GET_ANIM_VISUAL_LENGTH</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Show Voice Message</t>
+          <t>Get Animation Visual Length</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>语音对话</t>
+          <t>获取动画视觉时长</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>SHOW_VOICE_MESSAGE_DESC</t>
+          <t>GET_ANIM_VISUAL_LENGTH_DESC</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Play a non-spatial voice clip and show a dialogue message on the current map scene. refActorTag controls dialogue-window placement.</t>
+          <t>Get the visual duration of an animation, excluding sound track length (seconds).</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>在当前地图场景中播放非空间语音并显示对话。refActorTag 控制对话窗口位置。</t>
+          <t>获取指定动画的视觉时长（秒），不包含音轨长度。</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>SHOW_MESSAGE</t>
+          <t>TO_SHORT_NUMBER</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Show Message</t>
+          <t>Short Number</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>显示对话</t>
+          <t>数值缩写</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>SHOW_MESSAGE_DESC</t>
+          <t>TO_SHORT_NUMBER_DESC</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Show dialogue on the current map scene. refActorTag controls dialogue-window placement.</t>
+          <t>Shorten large numbers with k/m/b suffixes.</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>在当前地图场景中显示对话。refActorTag 用于控制对话窗口位置。</t>
+          <t>将较大的数字显示为 k/m/b 缩写。</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>SHOW_SELECTION</t>
+          <t>SHOW_VOICE_MESSAGE</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Show Selection</t>
+          <t>Show Voice Message</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>显示选项</t>
+          <t>语音对话</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>SHOW_SELECTION_DESC</t>
+          <t>SHOW_VOICE_MESSAGE_DESC</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Show a selection window on the current map scene. refActorTag controls selection-window placement.</t>
+          <t>Play a non-spatial voice clip and show a dialogue message on the current map scene. refActorTag controls dialogue-window placement.</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>在当前地图场景中显示选项窗口。refActorTag 用于控制选项窗口位置。</t>
+          <t>在当前地图场景中播放非空间语音并显示对话。refActorTag 控制对话窗口位置。</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>GET_PLAYER_ATTR_REF</t>
+          <t>SHOW_MESSAGE</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>Get Player Attribute Ref</t>
+          <t>Show Message</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>获取玩家属性引用</t>
+          <t>显示对话</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>GET_PLAYER_ATTR_REF_DESC</t>
+          <t>SHOW_MESSAGE_DESC</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Get a readable/writable reference to a player attribute (e.g. HP, ATK, DEF, GOLD).</t>
+          <t>Show dialogue on the current map scene. refActorTag controls dialogue-window placement.</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>获取玩家指定属性的可读写引用（如 HP/ATK/DEF/GOLD）。</t>
+          <t>在当前地图场景中显示对话。refActorTag 用于控制对话窗口位置。</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>ADD_HP</t>
+          <t>SHOW_SELECTION</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Add HP</t>
+          <t>Show Selection</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>增加HP</t>
+          <t>显示选项</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>ADD_HP_DESC</t>
+          <t>SHOW_SELECTION_DESC</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Add HP to the player (can be negative to subtract).</t>
+          <t>Show a selection window on the current map scene. refActorTag controls selection-window placement.</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>为玩家增加（或减少）HP。</t>
+          <t>在当前地图场景中显示选项窗口。refActorTag 用于控制选项窗口位置。</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>ADD_ATK</t>
+          <t>SHOW_REF_SELECTION</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Add ATK</t>
+          <t>Show Ref Selection</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>增加攻击力</t>
+          <t>显示引用选项</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>ADD_ATK_DESC</t>
+          <t>SHOW_REF_SELECTION_DESC</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Add ATK to the player (can be negative to subtract).</t>
+          <t>Show a selection window on the current map scene. Uses a direct actor reference for selection-window placement.</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>为玩家增加（或减少）攻击力。</t>
+          <t>在当前地图场景中显示选项窗口。通过直接 Actor 引用进行选项窗口定位。</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>ADD_DEF</t>
+          <t>GET_PLAYER_ATTR_REF</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Add DEF</t>
+          <t>Get Player Attribute Ref</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>增加防御力</t>
+          <t>获取玩家属性引用</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>ADD_DEF_DESC</t>
+          <t>GET_PLAYER_ATTR_REF_DESC</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Add DEF to the player (can be negative to subtract).</t>
+          <t>Get a readable/writable reference to a player attribute (e.g. HP, ATK, DEF, GOLD).</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>为玩家增加（或减少）防御力。</t>
+          <t>获取玩家指定属性的可读写引用（如 HP/ATK/DEF/GOLD）。</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>TONE_SHADER_LOAD_FAILED</t>
+          <t>ADD_HP</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Failed to load screen tone shader</t>
+          <t>Add HP</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>画面色调着色器加载失败</t>
+          <t>增加HP</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>CHANGE_SCREEN_TONE</t>
+          <t>ADD_HP_DESC</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Change Screen Tone</t>
+          <t>Add HP to the player (can be negative to subtract).</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>更改画面色调</t>
+          <t>为玩家增加（或减少）HP。</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>CHANGE_SCREEN_TONE_DESC</t>
+          <t>ADD_ATK</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Change the screen tone over time. Red, green, and blue range from -255 to 255; gray ranges from 0 to 255; duration is in seconds.</t>
+          <t>Add ATK</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>在指定时间内更改画面色调。红、绿、蓝范围为 -255 到 255；灰度范围为 0 到 255；持续时间单位为秒。</t>
+          <t>增加攻击力</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>CLEAR_SCREEN_TONE</t>
+          <t>ADD_ATK_DESC</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Clear Screen Tone</t>
+          <t>Add ATK to the player (can be negative to subtract).</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>清除画面色调</t>
+          <t>为玩家增加（或减少）攻击力。</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>CLEAR_SCREEN_TONE_DESC</t>
+          <t>ADD_DEF</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Fade the screen tone back to normal over the given duration in seconds.</t>
+          <t>Add DEF</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>在指定秒数内将画面色调恢复为正常。</t>
+          <t>增加防御力</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>CREATE_ACTOR_FROM_BP_PATH</t>
+          <t>ADD_DEF_DESC</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Create Actor From BP Path</t>
+          <t>Add DEF to the player (can be negative to subtract).</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>从蓝图路径创建 Actor</t>
+          <t>为玩家增加（或减少）防御力。</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>CREATE_ACTOR_FROM_BP_PATH_DESC</t>
+          <t>TONE_SHADER_LOAD_FAILED</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Create an actor from a blueprint class path and spawn it on the current map.</t>
+          <t>Failed to load screen tone shader</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>根据蓝图类路径创建 Actor，并生成到当前地图。</t>
+          <t>画面色调着色器加载失败</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>ADD_TIMER</t>
+          <t>CHANGE_SCREEN_TONE</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Add Timer</t>
+          <t>Change Screen Tone</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>添加计时器</t>
+          <t>更改画面色调</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>ADD_TIMER_DESC</t>
+          <t>CHANGE_SCREEN_TONE_DESC</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Wait for a scene timer. If blocking is enabled, player movement and scene hotkeys are disabled until TimeUp.</t>
+          <t>Change the screen tone over time. Red, green, and blue range from -255 to 255; gray ranges from 0 to 255; duration is in seconds.</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>等待场景计时器。如果启用阻塞，TimeUp 前玩家移动和场景快捷键不可用。</t>
+          <t>在指定时间内更改画面色调。红、绿、蓝范围为 -255 到 255；灰度范围为 0 到 255；持续时间单位为秒。</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>RECORD_DESTROYED_ACTOR</t>
+          <t>CLEAR_SCREEN_TONE</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Record Destroyed Actor</t>
+          <t>Clear Screen Tone</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>记录已销毁 Actor</t>
+          <t>清除画面色调</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>RECORD_DESTROYED_ACTOR_DESC</t>
+          <t>CLEAR_SCREEN_TONE_DESC</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Record a destroyed actor for persistence on the current map scene.</t>
+          <t>Fade the screen tone back to normal over the given duration in seconds.</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>在当前地图场景中记录一个已销毁 Actor，用于存档持久化。</t>
+          <t>在指定秒数内将画面色调恢复为正常。</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>SELF_RECORD_DESTROYED</t>
+          <t>CREATE_ACTOR_FROM_BP_PATH</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>Self Record Destroyed</t>
+          <t>Create Actor From BP Path</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>自身记录已销毁</t>
+          <t>从蓝图路径创建 Actor</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>SELF_RECORD_DESTROYED_DESC</t>
+          <t>CREATE_ACTOR_FROM_BP_PATH_DESC</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Record the blueprint owner as a destroyed actor for persistence on the current map scene.</t>
+          <t>Create an actor from a blueprint class path and spawn it on the current map.</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>将蓝图所有者记录为已销毁 Actor，用于在当前地图场景中持久化。</t>
+          <t>根据蓝图类路径创建 Actor，并生成到当前地图。</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>RECORD_AND_DESTROY_ACTOR</t>
+          <t>ADD_TIMER</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Record And Destroy Actor</t>
+          <t>Add Timer</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>记录并销毁 Actor</t>
+          <t>添加计时器</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>RECORD_AND_DESTROY_ACTOR_DESC</t>
+          <t>ADD_TIMER_DESC</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Record a destroyed actor for persistence and destroy it on the current map scene.</t>
+          <t>Wait for a scene timer. If blocking is enabled, player movement and scene hotkeys are disabled until TimeUp.</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>在当前地图场景中记录一个已销毁 Actor 并销毁它。</t>
+          <t>等待场景计时器。如果启用阻塞，TimeUp 前玩家移动和场景快捷键不可用。</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>SELF_RECORD_AND_DESTROY</t>
+          <t>RECORD_DESTROYED_ACTOR</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>Self Record And Destroy</t>
+          <t>Record Destroyed Actor</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>自身记录并销毁</t>
+          <t>记录已销毁 Actor</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>SELF_RECORD_AND_DESTROY_DESC</t>
+          <t>RECORD_DESTROYED_ACTOR_DESC</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>Record the blueprint owner as destroyed for persistence and destroy it on the current map scene.</t>
+          <t>Record a destroyed actor for persistence on the current map scene.</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>将蓝图所有者记录为已销毁并销毁它，用于在当前地图场景中持久化。</t>
+          <t>在当前地图场景中记录一个已销毁 Actor，用于存档持久化。</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>SHOW_REF_MESSAGE</t>
+          <t>SELF_RECORD_DESTROYED</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>Show Ref Message</t>
+          <t>Self Record Destroyed</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>显示引用消息</t>
+          <t>自身记录已销毁</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>SHOW_REF_MESSAGE_DESC</t>
+          <t>SELF_RECORD_DESTROYED_DESC</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Show a dialogue message on the current map scene. Uses a direct actor reference for window placement.</t>
+          <t>Record the blueprint owner as a destroyed actor for persistence on the current map scene.</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>在当前地图场景中显示对话，通过直接 Actor 引用进行窗口定位。</t>
+          <t>将蓝图所有者记录为已销毁 Actor，用于在当前地图场景中持久化。</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>SHOW_VOICE_REF_MESSAGE</t>
+          <t>RECORD_AND_DESTROY_ACTOR</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Show Voice Ref Message</t>
+          <t>Record And Destroy Actor</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>显示引用语音消息</t>
+          <t>记录并销毁 Actor</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>SHOW_VOICE_REF_MESSAGE_DESC</t>
+          <t>RECORD_AND_DESTROY_ACTOR_DESC</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Play a spatial voice clip and show a dialogue message on the current map scene. Uses a direct actor reference for voice positioning.</t>
+          <t>Record a destroyed actor for persistence and destroy it on the current map scene.</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>在当前地图场景中播放空间语音并显示对话。通过直接 Actor 引用进行语音定位。</t>
+          <t>在当前地图场景中记录一个已销毁 Actor 并销毁它。</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>GET_SELF_ATTR</t>
+          <t>SELF_RECORD_AND_DESTROY</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Get Self Attr</t>
+          <t>Self Record And Destroy</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>获取自身属性</t>
+          <t>自身记录并销毁</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>GET_SELF_ATTR_DESC</t>
+          <t>SELF_RECORD_AND_DESTROY_DESC</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Read an attribute value from the blueprint owner</t>
+          <t>Record the blueprint owner as destroyed for persistence and destroy it on the current map scene.</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>读取蓝图拥有者的属性值</t>
+          <t>将蓝图所有者记录为已销毁并销毁它，用于在当前地图场景中持久化。</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>SET_SELF_ATTR</t>
+          <t>SHOW_REF_MESSAGE</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Set Self Attr</t>
+          <t>Show Ref Message</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>设置自身属性</t>
+          <t>显示引用消息</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>SET_SELF_ATTR_DESC</t>
+          <t>SHOW_REF_MESSAGE_DESC</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Set an attribute value on the blueprint owner</t>
+          <t>Show a dialogue message on the current map scene. Uses a direct actor reference for window placement.</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>设置蓝图拥有者的属性值</t>
+          <t>在当前地图场景中显示对话，通过直接 Actor 引用进行窗口定位。</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>IF_PLAYER_OVERLAPS</t>
+          <t>SHOW_VOICE_REF_MESSAGE</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>If Player Overlaps</t>
+          <t>Show Voice Ref Message</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>玩家是否重叠</t>
+          <t>显示引用语音消息</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>IF_PLAYER_OVERLAPS_DESC</t>
+          <t>SHOW_VOICE_REF_MESSAGE_DESC</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>Check if the player shares the same cell as the blueprint owner</t>
+          <t>Play a spatial voice clip and show a dialogue message on the current map scene. Uses a direct actor reference for voice positioning.</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>判断玩家是否与蓝图拥有者处于同一格子</t>
+          <t>在当前地图场景中播放空间语音并显示对话。通过直接 Actor 引用进行语音定位。</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>IF_GAME_VAR</t>
+          <t>GET_SELF_ATTR</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>If Game Var</t>
+          <t>Get Self Attr</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>判断游戏变量</t>
+          <t>获取自身属性</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>IF_GAME_VAR_DESC</t>
+          <t>GET_SELF_ATTR_DESC</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Compare a game variable with a given value, returning a true/false branch</t>
+          <t>Read an attribute value from the blueprint owner</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>将游戏变量与给定值进行比较，返回真假分支</t>
+          <t>读取蓝图拥有者的属性值</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>GET_ACTOR_BY_TAG</t>
+          <t>SET_SELF_ATTR</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Get Actor By Tag</t>
+          <t>Set Self Attr</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>按标签查找角色</t>
+          <t>设置自身属性</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>GET_ACTOR_BY_TAG_DESC</t>
+          <t>SET_SELF_ATTR_DESC</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>Find an actor by tag on the current map</t>
+          <t>Set an attribute value on the blueprint owner</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>在当前地图上按标签查找角色</t>
+          <t>设置蓝图拥有者的属性值</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>GET_ALL_ACTORS</t>
+          <t>IF_PLAYER_OVERLAPS</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Get All Actors</t>
+          <t>If Player Overlaps</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>获取全部角色</t>
+          <t>玩家是否重叠</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
+          <t>IF_PLAYER_OVERLAPS_DESC</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Check if the player shares the same cell as the blueprint owner</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>判断玩家是否与蓝图拥有者处于同一格子</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>IF_GAME_VAR</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>If Game Var</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>判断游戏变量</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>IF_GAME_VAR_DESC</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Compare a game variable with a given value, returning a true/false branch</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>将游戏变量与给定值进行比较，返回真假分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>GET_ACTOR_BY_TAG</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Get Actor By Tag</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>按标签查找角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>GET_ACTOR_BY_TAG_DESC</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Find an actor by tag on the current map</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>在当前地图上按标签查找角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>GET_ALL_ACTORS</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Get All Actors</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>获取全部角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
           <t>GET_ALL_ACTORS_DESC</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr">
+      <c r="B459" t="inlineStr">
         <is>
           <t>Get a list of all actors on the current map</t>
         </is>
       </c>
-      <c r="C453" t="inlineStr">
+      <c r="C459" t="inlineStr">
         <is>
           <t>获取当前地图上的所有角色列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>REDUCE_STATE_FROM</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Reduce State From</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>减少战斗者状态层数</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>REDUCE_STATE_FROM_DESC</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Reduce a state stack count on any battler. Remove the state when stacks reach zero.</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>减少任意战斗者身上的状态层数，层数归零时移除状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>REDUCE_PLAYER_STATE</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Reduce Player State</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>减少玩家状态层数</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>REDUCE_PLAYER_STATE_DESC</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Reduce a state stack count on the player. Remove the state when stacks reach zero.</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>减少玩家身上的状态层数，层数归零时移除状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>REMOVE_PLAYER_STATE</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Remove Player State</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>移除玩家状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>REMOVE_PLAYER_STATE_DESC</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Remove a state from the player.</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>移除玩家身上的指定状态。</t>
         </is>
       </c>
     </row>
@@ -8936,7 +9140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.75" customWidth="1" min="1" max="1"/>
@@ -9264,6 +9468,142 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>可以破坏面前的一块冰墙。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>POISONED_EASE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Antidote</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>解毒剂</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>POISONED_EASE_DESC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>It can reduce the accumulation of poison layers by 5 points.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>可以减少5点中毒层数累积。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>POISONED_RELEASE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Antitoxic</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>解毒药水</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>POISONED_RELEASE_DESC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>It can completely cure the poisoning state.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>可以完全解除中毒状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>WEAK_EASE</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Adrenaline</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>解衰剂</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>WEAK_EASE_DESC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>It can reduce the accumulation of 5 points of weakened layers.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>可以减少5点衰弱层数累积。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>WEAK_RELEASE</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Aqua-vitae</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>解衰药水</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>WEAK_RELEASE_DESC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>It can completely relieve the weakened state.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>可以完全解除衰弱状态。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update code structure, meta and shop
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,26 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="UI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Enemies" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Equips" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Classes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="States" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MapNames" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Specials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Player" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_1" localSheetId="0">System!$A$6:$C$249</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -30,17 +26,12 @@
   <fonts count="2">
     <font>
       <name val="等线"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="等线"/>
-      <charset val="134"/>
-      <family val="3"/>
       <sz val="9"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -53,32 +44,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -151,7 +134,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -193,74 +176,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -272,23 +195,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -298,23 +221,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -322,26 +245,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -376,17 +296,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -401,13 +321,6 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -417,12 +330,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C465"/>
+  <dimension ref="A1:C469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col width="38.75" customWidth="1" min="1" max="1"/>
-    <col width="61.83203125" customWidth="1" min="2" max="2"/>
-    <col width="52.33203125" customWidth="1" min="3" max="3"/>
+    <col width="38.75" customWidth="1" style="1" min="1" max="1"/>
+    <col width="61.83203125" customWidth="1" style="1" min="2" max="2"/>
+    <col width="52.33203125" customWidth="1" style="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4494,12 +4407,12 @@
           <t>IADD</t>
         </is>
       </c>
-      <c r="B240" s="1" t="inlineStr">
+      <c r="B240" t="inlineStr">
         <is>
           <t>+=</t>
         </is>
       </c>
-      <c r="C240" s="1" t="inlineStr">
+      <c r="C240" t="inlineStr">
         <is>
           <t>+=</t>
         </is>
@@ -4528,12 +4441,12 @@
           <t>ISUB</t>
         </is>
       </c>
-      <c r="B242" s="1" t="inlineStr">
+      <c r="B242" t="inlineStr">
         <is>
           <t>-=</t>
         </is>
       </c>
-      <c r="C242" s="1" t="inlineStr">
+      <c r="C242" t="inlineStr">
         <is>
           <t>-=</t>
         </is>
@@ -4562,12 +4475,12 @@
           <t>IMUL</t>
         </is>
       </c>
-      <c r="B244" s="1" t="inlineStr">
+      <c r="B244" t="inlineStr">
         <is>
           <t>*=</t>
         </is>
       </c>
-      <c r="C244" s="1" t="inlineStr">
+      <c r="C244" t="inlineStr">
         <is>
           <t>*=</t>
         </is>
@@ -4596,12 +4509,12 @@
           <t>IDIV</t>
         </is>
       </c>
-      <c r="B246" s="1" t="inlineStr">
+      <c r="B246" t="inlineStr">
         <is>
           <t>/=</t>
         </is>
       </c>
-      <c r="C246" s="1" t="inlineStr">
+      <c r="C246" t="inlineStr">
         <is>
           <t>/=</t>
         </is>
@@ -4664,12 +4577,12 @@
           <t>IPOW</t>
         </is>
       </c>
-      <c r="B250" s="1" t="inlineStr">
+      <c r="B250" t="inlineStr">
         <is>
           <t>**=</t>
         </is>
       </c>
-      <c r="C250" s="1" t="inlineStr">
+      <c r="C250" t="inlineStr">
         <is>
           <t>**=</t>
         </is>
@@ -8330,9 +8243,76 @@
         </is>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>OPEN_ATTR_SHOP</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Open Attribute Shop</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>打开数值商店</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>OPEN_ATTR_SHOP_DESC</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Opens an attribute shop using an Actor reference for the shop avatar.</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>使用 Actor 引用作为商店头像，打开数值商店。</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>OPEN_ATTR_SHOP_BY_TAG</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Open Attribute Shop By Tag</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>按标签打开数值商店</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>OPEN_ATTR_SHOP_BY_TAG_DESC</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Finds a map Actor by tag and opens an attribute shop using it as the shop avatar.</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>按标签查找地图 Actor，并将其作为商店头像打开数值商店。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -8397,7 +8377,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -8407,12 +8387,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col width="17.4140625" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="17.25" customWidth="1" min="3" max="3"/>
+    <col width="17.4140625" customWidth="1" style="1" min="1" max="1"/>
+    <col width="18" customWidth="1" style="1" min="2" max="2"/>
+    <col width="17.25" customWidth="1" style="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8979,153 +8959,68 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>STAT_HP</t>
+          <t>SHOP_ATTR_LEAVE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HP:</t>
+          <t>Leave</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>生命:</t>
+          <t>离开</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>STAT_MAXHP</t>
+          <t>SHOP_ATTR_PRICE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MAXHP:</t>
+          <t>Current Price ({gold})</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>最大生命:</t>
+          <t>当前价格（{gold}）</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>STAT_ATK</t>
+          <t>SHOP_NAME</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ATK:</t>
+          <t>The Gold of Avarice</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>攻击:</t>
+          <t>贪婪之神</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>STAT_DEF</t>
+          <t>SHOP_DESC</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DEF:</t>
+          <t>How insignificant are humankind! \nIf you offer me enough wealth, \nI will grant you a certain amount of power!</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>防御:</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>STAT_EXP</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>EXP:</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>经验:</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>STAT_GOLD</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>GOLD:</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>金币:</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>STAT_DMG</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>DMG:</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>伤害:</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>STAT_HIT</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>HIT:</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>连击:</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>STAT_CRIT</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>CRIT:</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>临界:</t>
+          <t>渺小的人类啊。\n如果你向我献上财富，\n我会给予你一定的力量！</t>
         </is>
       </c>
     </row>
@@ -9143,9 +9038,9 @@
   <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col width="25.75" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="24.83203125" customWidth="1" min="3" max="3"/>
+    <col width="25.75" customWidth="1" style="1" min="1" max="1"/>
+    <col width="29" customWidth="1" style="1" min="2" max="2"/>
+    <col width="24.83203125" customWidth="1" style="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9609,7 +9504,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -9622,9 +9516,9 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col width="29.58203125" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="32.33203125" customWidth="1" min="3" max="3"/>
+    <col width="29.58203125" customWidth="1" style="1" min="1" max="1"/>
+    <col width="29" customWidth="1" style="1" min="2" max="2"/>
+    <col width="32.33203125" customWidth="1" style="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9948,7 +9842,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -10013,7 +9907,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -10129,7 +10023,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -10194,7 +10088,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -10463,6 +10357,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update editor, bp and animation
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -331,7 +331,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C469"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="38.75" customWidth="1" style="1" min="1" max="1"/>
     <col width="61.83203125" customWidth="1" style="1" min="2" max="2"/>
@@ -8387,8 +8387,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <dimension ref="A1:C39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="17.4140625" customWidth="1" style="1" min="1" max="1"/>
     <col width="18" customWidth="1" style="1" min="2" max="2"/>
@@ -9021,6 +9021,40 @@
       <c r="C37" t="inlineStr">
         <is>
           <t>渺小的人类啊。\n如果你向我献上财富，\n我会给予你一定的力量！</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>EXP_SHOP_NAME</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>The Gold of War</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>战斗之神</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EXP_SHOP_DESC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Offer thy hard-won essence, O hero of mortality! \nAnd I shall transform it into thy strength.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>献上经验吧，英雄的人类！\n我会将经验转换成你的力量！</t>
         </is>
       </c>
     </row>
@@ -9036,7 +9070,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="25.75" customWidth="1" style="1" min="1" max="1"/>
     <col width="29" customWidth="1" style="1" min="2" max="2"/>
@@ -9514,7 +9548,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14" outlineLevelCol="0"/>
   <cols>
     <col width="29.58203125" customWidth="1" style="1" min="1" max="1"/>
     <col width="29" customWidth="1" style="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Update AI, details, equip UI, editor and docs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -330,7 +330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C471"/>
+  <dimension ref="A1:C477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" style="1" min="1" max="1"/>
@@ -8342,6 +8342,108 @@
       <c r="C471" t="inlineStr">
         <is>
           <t>按标签查找到地图Actor，并启用或禁用其移动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>CREATE_DICT</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Create Dict</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>创建字典</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>CREATE_DICT_DESC</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Create a new empty dict.</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>创建一个新的空字典。</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>CREATE_LIST</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Create List</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>创建列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>CREATE_LIST_DESC</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Create a new empty list.</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>创建一个新的空列表。</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>SET_AUTO_PATH_TO_DESTINATION_BY_TAG</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>按标签自动寻路到终点</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Set Auto Path to Destination By Tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>SET_AUTO_PATH_TO_DESTINATION_BY_TAG_DESC</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>按标签找到地图 Actor 并自动寻路到指定地图格。Started 出口立即继续；Finished 在移动结束后继续。</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Finds a map Actor by tag and pathfinds it to the target map cell. Started continues immediately; Finished continues after movement ends.</t>
         </is>
       </c>
     </row>
@@ -9289,12 +9391,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>You can teleport to the map you had been to with it(Hotkey: F).</t>
+          <t>You can teleport to the map you had been to with it(Hotkey: G).</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>持有后可以在前往过的传送点（快捷键F）。</t>
+          <t>持有后可以在前往过的传送点（快捷键G）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update bp editor and some bps
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -330,7 +330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C477"/>
+  <dimension ref="A1:C585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" style="1" min="1" max="1"/>
@@ -8444,6 +8444,1842 @@
       <c r="C477" t="inlineStr">
         <is>
           <t>Finds a map Actor by tag and pathfinds it to the target map cell. Started continues immediately; Finished continues after movement ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>CREATE_ACTOR_FROM_BP_PATH_WITH_DEFAULTS</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Create Actor From BP Path With Defaults</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>按蓝图路径创建 Actor（带默认值）</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>CREATE_ACTOR_FROM_BP_PATH_WITH_DEFAULTS_DESC</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Create an actor from a blueprint class path, apply defaults overrides, and spawn it on the current map.</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>按蓝图类路径创建 Actor，先应用 defaults 字典中的类默认属性覆盖，再生成到当前地图。</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_TAG</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>标签</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_TAG_DESC</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Identifier used to find this actor on a map.</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>用于在地图上查找该 Actor 的标识。</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_SWITCH_INTERVAL</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Frame Interval</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>帧切换间隔</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_SWITCH_INTERVAL_DESC</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Sprite animation frame interval in seconds.</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>精灵动画帧切换间隔，单位为秒。</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_ANIMATABLE</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Animatable</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>启用动画</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_ANIMATABLE_DESC</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Whether sprite-sheet animation is enabled.</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>是否启用精灵表动画。</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_MATERIAL</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>材质</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_MATERIAL_DESC</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Surface material settings used by movement, opacity, and lighting.</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>用于移动、透明度和光照的表面材质设置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_SHADER_PATH</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Shader Path</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>着色器路径</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_SHADER_PATH_DESC</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Fragment shader path under Assets/Shaders.</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Assets/Shaders 下的片段着色器路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_COLLISION_ENABLED</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Collision Enabled</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>启用碰撞</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_COLLISION_ENABLED_DESC</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Whether this actor blocks movement.</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>该 Actor 是否阻挡移动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_TICKABLE</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Tickable</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>启用 Tick</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_TICKABLE_DESC</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Whether tick events are dispatched every frame.</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>是否每帧分发 Tick 事件。</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_SPEED</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Move Speed</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>移动速度</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_SPEED_DESC</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Movement speed in pixels per second.</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>移动速度，单位为像素/秒。</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_AUTO_SOUND</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Auto Sound</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>自动音效</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_AUTO_SOUND_DESC</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Sound asset under Assets/Sounds played automatically as spatial audio.</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Assets/Sounds 下自动播放的音效素材，会作为空间音频播放。</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_AUTO_SOUND_INTERVAL</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Auto Sound Interval</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>自动音效间隔</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_AUTO_SOUND_INTERVAL_DESC</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Delay from one automatic sound ending to the next playback start.</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>一次自动音效播放结束后，到下一次开始播放前的等待时间。</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_AUTO_SOUND_PARAMS</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Auto Sound Params</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>自动音效参数</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_AUTO_SOUND_PARAMS_DESC</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Nested spatial sound parameters used by the automatic sound.</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>自动音效使用的嵌套空间音频参数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_TEXTURE_PATH</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Texture Path</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>纹理路径</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_TEXTURE_PATH_DESC</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Character texture asset path under Assets/Characters.</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Assets/Characters 下的角色纹理素材路径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_RECT</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Default Rect</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>默认矩形</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_RECT_DESC</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Default texture rectangle stored as origin and size.</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>默认贴图矩形，以起点和尺寸保存。</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Default Translation</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>默认偏移</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_TRANSLATION_DESC</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Default position offset on the actor sprite.</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Actor 精灵的默认位置偏移。</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_ROTATION</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Default Rotation</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>默认旋转</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_ROTATION_DESC</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Default rotation in degrees.</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>默认旋转角度，单位为度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_SCALE</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Default Scale</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>默认缩放</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_SCALE_DESC</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Default x/y scale factors.</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>默认 x/y 缩放比例。</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_ORIGIN</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Default Origin</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>默认原点</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_DEFAULT_ORIGIN_DESC</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Default origin point for transformations.</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>用于变换的默认原点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_LIGHT_COMP</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Light Component</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>光照组件</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_LIGHT_COMP_DESC</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Optional self-light settings attached to this actor.</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>附加到该 Actor 的可选自发光设置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_CHILD_ACTOR_COMP</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Child Actor Component</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>子 Actor 组件</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_CHILD_ACTOR_COMP_DESC</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Optional child actor spawned relative to this actor.</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>相对该 Actor 生成的可选子 Actor。</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>AUTO_SOUND_VAR_VOLUME</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>音量</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>AUTO_SOUND_VAR_VOLUME_DESC</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Base sound volume before global sound-volume scaling.</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>应用全局音效音量前的基础音量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>AUTO_SOUND_VAR_MIN_DISTANCE</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Min Distance</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>最小距离</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>AUTO_SOUND_VAR_MIN_DISTANCE_DESC</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Distance where the sound remains at full volume.</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>声音保持最大音量的距离。</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>AUTO_SOUND_VAR_ATTENUATION</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Attenuation</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>衰减</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>AUTO_SOUND_VAR_ATTENUATION_DESC</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Distance fade factor for the automatic sound.</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>自动音效的距离衰减系数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>CHARACTER_VAR_DIRECTION</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>朝向</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>CHARACTER_VAR_DIRECTION_DESC</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Current facing direction.</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>当前面向的方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>CHARACTER_VAR_DIRECTION_FIX</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Direction Fix</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>固定朝向</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>CHARACTER_VAR_DIRECTION_FIX_DESC</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>If enabled, movement will not update the facing direction.</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>启用后，移动不会更新朝向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>CHARACTER_VAR_ANIMATE_WITHOUT_MOVING</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Animate While Idle</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>静止时播放动画</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>CHARACTER_VAR_ANIMATE_WITHOUT_MOVING_DESC</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>If enabled, the character animation plays even when idle.</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>启用后，即使角色静止也会播放动画。</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>CHILD_ACTOR_COMP_VAR_CLASS_NAME</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Class Name</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>类名</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>CHILD_ACTOR_COMP_VAR_CLASS_NAME_DESC</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Actor class path or generated blueprint class name to spawn.</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>要生成的 Actor 类路径或生成的蓝图类名。</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>CHILD_ACTOR_COMP_VAR_RELATIVE_POSITION</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Relative Position</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>相对位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>CHILD_ACTOR_COMP_VAR_RELATIVE_POSITION_DESC</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Spawn offset relative to the parent actor.</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>相对父 Actor 的生成偏移。</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>LIGHT_COMP_VAR_LIGHT_COLOUR</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Light Colour</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>光照颜色</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>LIGHT_COMP_VAR_LIGHT_COLOUR_DESC</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Self-light colour stored as RGBA.</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>以 RGBA 保存的自发光颜色。</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>LIGHT_COMP_VAR_LIGHT_RADIUS</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Light Radius</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>光照半径</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>LIGHT_COMP_VAR_LIGHT_RADIUS_DESC</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Self-light radius in pixels.</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>自发光半径，单位为像素。</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>INFO_VAR_ID</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>INFO_VAR_ID_DESC</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Unique identifier for this info object.</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>该信息对象的唯一标识。</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>GAME_MAP_VAR_DEFAULT_COVER_ALPHA</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Default Cover Alpha</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>默认遮罩透明度</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>GAME_MAP_VAR_DEFAULT_COVER_ALPHA_DESC</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Default alpha used by cover and occlusion rendering.</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>遮罩和遮挡渲染使用的默认透明度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>GAME_MAP_VAR_MAP_VIEW_OFFSET</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Map View Offset</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>地图视图偏移</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>GAME_MAP_VAR_MAP_VIEW_OFFSET_DESC</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Default camera/view offset for map presentation.</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>地图显示使用的默认镜头/视图偏移。</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_LOOP</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Loop</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>循环</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_LOOP_DESC</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Whether to loop playback.</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>是否循环播放。</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_OFFSET</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Offset</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>播放偏移</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_OFFSET_DESC</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Playback offset in seconds or a Time value.</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>播放偏移，可为秒数或 Time 值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_NEED_EFFECT</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Need Effect</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>需要效果器</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_NEED_EFFECT_DESC</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Whether a sound effect processor is required.</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>是否需要音效处理器。</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_SOUND_EFFECT</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Sound Effect</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>音效处理器</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_SOUND_EFFECT_DESC</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Custom effect processor callback.</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>自定义音效处理回调。</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_PITCH</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Pitch</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>音调</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_PITCH_DESC</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Pitch multiplier, where 1.0 is normal.</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>音调倍率，1.0 为正常。</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_PAN</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Pan</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>声像</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_PAN_DESC</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Stereo pan from -1.0 left to 1.0 right.</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>立体声声像，-1.0 为左，1.0 为右。</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_VOLUME</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>音量</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_VOLUME_DESC</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Volume from 0.0 mute to 100.0 maximum.</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>音量，0.0 为静音，100.0 为最大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_SPATIAL</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Spatial</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>空间音频</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_SPATIAL_DESC</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Whether spatialisation is enabled.</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>是否启用空间化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_POSITION</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_POSITION_DESC</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Sound position in 3D space.</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>声音在 3D 空间中的位置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_DIRECTION</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_DIRECTION_DESC</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Sound direction in 3D space.</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>声音在 3D 空间中的方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_CONE</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Cone</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>声锥</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_CONE_DESC</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Attenuation cone settings.</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>声源方向衰减锥设置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_VELOCITY</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Velocity</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>速度</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_VELOCITY_DESC</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Sound source velocity used for Doppler.</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>用于多普勒效果的声源速度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_DOPPLER_FACTOR</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Doppler Factor</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>多普勒系数</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_DOPPLER_FACTOR_DESC</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Doppler effect factor.</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>多普勒效果系数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_DIRECTIONAL_ATTENUATION_FACTOR</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Directional Attenuation</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>方向衰减</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_DIRECTIONAL_ATTENUATION_FACTOR_DESC</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Directional attenuation factor.</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>方向性衰减系数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_RELATIVE_TO_LISTENER</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Relative To Listener</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>相对监听者</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_RELATIVE_TO_LISTENER_DESC</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Whether the position is relative to the listener.</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>位置是否相对监听者。</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MIN_DISTANCE</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Min Distance</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>最小距离</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MIN_DISTANCE_DESC</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Minimum attenuation distance.</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>开始衰减前的最小距离。</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MAX_DISTANCE</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Max Distance</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>最大距离</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MAX_DISTANCE_DESC</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Maximum attenuation distance.</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>最大衰减距离。</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MIN_GAIN</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Min Gain</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>最小增益</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MIN_GAIN_DESC</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Minimum gain after attenuation.</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>衰减后的最小增益。</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MAX_GAIN</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Max Gain</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>最大增益</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_MAX_GAIN_DESC</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Maximum gain after attenuation.</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>衰减后的最大增益。</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_ATTENUATION</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Attenuation</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>衰减</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>SOUND_FILTER_VAR_ATTENUATION_DESC</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Distance attenuation factor.</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>距离衰减系数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>MUSIC_FILTER_VAR_LOOP_POINT</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Loop Point</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>循环点</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>MUSIC_FILTER_VAR_LOOP_POINT_DESC</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Optional loop time range for music.</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>音乐可选的循环时间范围。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update editor layout, C ext and docs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -353,7 +353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C585"/>
+  <dimension ref="A1:C589"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -10303,6 +10303,74 @@
       <c r="C585" t="inlineStr">
         <is>
           <t>音乐可选的循环时间范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>FOR_LOOP</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>For Loop</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>For 循环</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>FOR_LOOP_DESC</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Loop from firstIndex to lastIndex inclusively by step. LoopBody continues for each iteration, and Completed continues after the loop. Latent nodes are not currently supported inside the loop body.</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>从 firstIndex 到 lastIndex 按 step 闭区间循环。LoopBody 每轮继续，Completed 在循环结束后继续。循环体暂不支持 latent 节点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>FOR_EACH</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>For Each</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>For Each</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>FOR_EACH_DESC</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Iterate over a list. LoopBody continues once for each element and outputs element and index; Completed continues after iteration. Latent nodes are not currently supported inside the loop body.</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>遍历列表。LoopBody 每个元素继续一次，并输出 element 与 index；Completed 在遍历结束后继续。循环体暂不支持 latent 节点。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update packing, specials and general data enums
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -10385,7 +10385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <sheetData>
     <row r="1">
@@ -10640,6 +10640,108 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>持有者的攻击力视为不低于对方攻击力。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>S_DOMAIN</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>领域</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>S_DOMAIN_DESC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>After each player move, the holder deals one-round damage while the player is within its Manhattan range.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>玩家每次移动后，若处于持有者的曼哈顿领域范围内，持有者造成一次单回合伤害。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>S_FLANK</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Flank</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>夹击</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S_FLANK_DESC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>After each player move, two opposite adjacent holders both deal one-round damage.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>玩家每次移动后，若被两个正对相邻的持有者夹在中间，二者各造成一次单回合伤害。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S_BLOCKADE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Blockade</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>阻击</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S_BLOCKADE_DESC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>After each player move, an adjacent holder deals one-round damage, retreats one cell away, and records its map position.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>玩家每次移动后，相邻的持有者造成一次单回合伤害，向远离玩家方向后退一格，并记录地图坐标。</t>
         </is>
       </c>
     </row>
@@ -10719,7 +10821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="17.4140625" customWidth="1" min="1" max="1"/>
@@ -11002,389 +11104,372 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MENU_LOAD</t>
+          <t>CONFIG_MIND_RESTART</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Load File</t>
+          <t>The configuration will take effect after a restart.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>读档</t>
+          <t>配置将在重启后生效</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CONFIG_MIND_RESTART</t>
+          <t>SHOP_BUY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The configuration will take effect after a restart.</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>配置将在重启后生效</t>
+          <t>购买</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SHOP_BUY</t>
+          <t>SHOP_SELL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>购买</t>
+          <t>出售</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SHOP_SELL</t>
+          <t>POINT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sell</t>
+          <t>P {index}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>出售</t>
+          <t>点位 {index}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>POINT</t>
+          <t>language</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>P {index}</t>
+          <t>Language</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>点位 {index}</t>
+          <t>语言</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>scale</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Scale</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>语言</t>
+          <t>缩放</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>scale</t>
+          <t>framerate</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Scale</t>
+          <t>Frame Rate</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>缩放</t>
+          <t>帧率</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>framerate</t>
+          <t>verticalsync</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Frame Rate</t>
+          <t>Vertical Sync</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>帧率</t>
+          <t>垂直同步</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>verticalsync</t>
+          <t>musicon</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Vertical Sync</t>
+          <t>Music</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>垂直同步</t>
+          <t>音乐</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>musicon</t>
+          <t>musicvolume</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Music Volume</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>音乐</t>
+          <t>音乐音量</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>musicvolume</t>
+          <t>soundon</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Music Volume</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>音乐音量</t>
+          <t>音效</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>soundon</t>
+          <t>soundvolume</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Sound Volume</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>音效</t>
+          <t>音效音量</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>soundvolume</t>
+          <t>voiceon</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sound Volume</t>
+          <t>Voice</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>音效音量</t>
+          <t>语音</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>voiceon</t>
+          <t>voicevolume</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Voice</t>
+          <t>Voice Volume</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>语音</t>
+          <t>语音音量</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>voicevolume</t>
+          <t>en_GB</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Voice Volume</t>
+          <t>English</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>语音音量</t>
+          <t>英语</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>en_GB</t>
+          <t>zh_CN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Simplified Chinese</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>英语</t>
+          <t>简体中文</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>zh_CN</t>
+          <t>SHOP_ATTR_LEAVE</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Simplified Chinese</t>
+          <t>Leave</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>简体中文</t>
+          <t>离开</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SHOP_ATTR_LEAVE</t>
+          <t>SHOP_ATTR_PRICE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Leave</t>
+          <t>Current Price ({gold})</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>离开</t>
+          <t>当前价格（{gold}）</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SHOP_ATTR_PRICE</t>
+          <t>SHOP_NAME</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Current Price ({gold})</t>
+          <t>The Gold of Avarice</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>当前价格（{gold}）</t>
+          <t>贪婪之神</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SHOP_NAME</t>
+          <t>SHOP_DESC</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>The Gold of Avarice</t>
+          <t>How insignificant are humankind! \nIf you offer me enough wealth, \nI will grant you a certain amount of power!</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>贪婪之神</t>
+          <t>渺小的人类啊。\n如果你向我献上财富，\n我会给予你一定的力量！</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SHOP_DESC</t>
+          <t>EXP_SHOP_NAME</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>How insignificant are humankind! \nIf you offer me enough wealth, \nI will grant you a certain amount of power!</t>
+          <t>The Gold of War</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>渺小的人类啊。\n如果你向我献上财富，\n我会给予你一定的力量！</t>
+          <t>战斗之神</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>EXP_SHOP_NAME</t>
+          <t>EXP_SHOP_DESC</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>The Gold of War</t>
+          <t>Offer thy hard-won essence, O hero of mortality! \nAnd I shall transform it into thy strength.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
-        <is>
-          <t>战斗之神</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>EXP_SHOP_DESC</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Offer thy hard-won essence, O hero of mortality! \nAnd I shall transform it into thy strength.</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
         <is>
           <t>献上经验吧，英雄的人类！\n我会将经验转换成你的力量！</t>
         </is>

</xml_diff>

<commit_message>
Update editor, hue, AI, plugin hooks and docs
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-31630" yWindow="2260" windowWidth="28800" windowHeight="15370" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="System" sheetId="1" state="visible" r:id="rId1"/>
@@ -353,7 +353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C589"/>
+  <dimension ref="A1:C591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="38.75" customWidth="1" min="1" max="1"/>
@@ -10371,6 +10371,40 @@
       <c r="C589" t="inlineStr">
         <is>
           <t>遍历列表。LoopBody 每个元素继续一次，并输出 element 与 index；Completed 在遍历结束后继续。循环体暂不支持 latent 节点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_HUE</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Hue</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>色相</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>ACTOR_VAR_HUE_DESC</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Hue rotation in degrees applied to this actor sprite. 0 keeps the original colour; values wrap every 360 degrees.</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>应用到该 Actor 精灵的色相旋转角度。0 保持原色；数值每 360 度循环。</t>
         </is>
       </c>
     </row>
@@ -12165,7 +12199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="29.58203125" customWidth="1" min="1" max="1"/>
@@ -12391,6 +12425,108 @@
       <c r="C13" t="inlineStr">
         <is>
           <t>这是一位骑士。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>WIZARD</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Wizard</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>巫师</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>WIZARD_DESC</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>This is a wizard.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>这是一个巫师。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>WHITE_KING</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>White King</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>魔法警卫</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>WHITE_KING_DESC</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>This is a white king.</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>这是一个魔法警卫。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BIG_WIZARD</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Big Wizard</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>大法师</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>BIG_WIZARD_DESC</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>This is a big wizard.</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>这是一个大法师。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update inst structure, animations and reborn special
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Other\Ludork\Sample\Data\Locale\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB3AF306-5407-46E7-88F6-865206C82966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B02A8BF-1E70-4343-B9E8-65FC89320410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5150" yWindow="3810" windowWidth="25260" windowHeight="14150" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="890" windowWidth="38420" windowHeight="19620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="468">
   <si>
     <t>ID</t>
   </si>
@@ -1060,12 +1060,6 @@
     <t>S_HARD_DESC</t>
   </si>
   <si>
-    <t>The holder's DEF is treated as at least the opponent's ATK minus 1 during damage calculation.</t>
-  </si>
-  <si>
-    <t>计算伤害时，持有者的防御力视为不低于对方攻击力-1。</t>
-  </si>
-  <si>
     <t>S_MAGIC</t>
   </si>
   <si>
@@ -1078,12 +1072,6 @@
     <t>S_MAGIC_DESC</t>
   </si>
   <si>
-    <t>During battle, the holder treats the opponent's DEF as 0 when calculating damage.</t>
-  </si>
-  <si>
-    <t>战斗中计算伤害时，持有者将对方防御力视为0。</t>
-  </si>
-  <si>
     <t>S_MULTIHIT</t>
   </si>
   <si>
@@ -1096,12 +1084,6 @@
     <t>S_MULTIHIT_DESC</t>
   </si>
   <si>
-    <t>During battle, each round's base damage is multiplied by the holder's hit count.</t>
-  </si>
-  <si>
-    <t>战斗中，持有者每回合基础伤害会按连击数倍计算。</t>
-  </si>
-  <si>
     <t>S_COMPETE</t>
   </si>
   <si>
@@ -1114,12 +1096,6 @@
     <t>S_COMPETE_DESC</t>
   </si>
   <si>
-    <t>The holder's ATK is treated as at least the opponent's ATK.</t>
-  </si>
-  <si>
-    <t>持有者的攻击力视为不低于对方攻击力。</t>
-  </si>
-  <si>
     <t>S_DOMAIN</t>
   </si>
   <si>
@@ -1132,12 +1108,6 @@
     <t>S_DOMAIN_DESC</t>
   </si>
   <si>
-    <t>After each player move, the holder deals one-round damage while the player is within its Manhattan range.</t>
-  </si>
-  <si>
-    <t>玩家每次移动后，若处于持有者的曼哈顿领域范围内，持有者造成一次单回合伤害。</t>
-  </si>
-  <si>
     <t>S_FLANK</t>
   </si>
   <si>
@@ -1150,12 +1120,6 @@
     <t>S_FLANK_DESC</t>
   </si>
   <si>
-    <t>After each player move, two opposite adjacent holders both deal one-round damage.</t>
-  </si>
-  <si>
-    <t>玩家每次移动后，若被两个正对相邻的持有者夹在中间，二者各造成一次单回合伤害。</t>
-  </si>
-  <si>
     <t>S_BLOCKADE</t>
   </si>
   <si>
@@ -1168,12 +1132,6 @@
     <t>S_BLOCKADE_DESC</t>
   </si>
   <si>
-    <t>After each player move, an adjacent holder deals one-round damage, retreats one cell away, and records its map position.</t>
-  </si>
-  <si>
-    <t>玩家每次移动后，相邻的持有者造成一次单回合伤害，向远离玩家方向后退一格，并记录地图坐标。</t>
-  </si>
-  <si>
     <t>BRAVOR</t>
   </si>
   <si>
@@ -1462,6 +1420,96 @@
   </si>
   <si>
     <t>You can teleport to the lower floor with it.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>S_REBORN</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>重生</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reborn</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>S_REBORN_DESC</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>The enemy's DEF is treated as at least the opponent's ATK minus 1 during damage calculation.</t>
+  </si>
+  <si>
+    <t>During battle, the enemy treats the opponent's DEF as 0 when calculating damage.</t>
+  </si>
+  <si>
+    <t>During battle, each round's base damage is multiplied by the enemy's hit count.</t>
+  </si>
+  <si>
+    <t>The enemy's ATK is treated as at least the opponent's ATK.</t>
+  </si>
+  <si>
+    <t>After each player move, the enemy deals one-round damage while the player is within its Manhattan range.</t>
+  </si>
+  <si>
+    <t>After each player move, two opposite adjacent enemys both deal one-round damage.</t>
+  </si>
+  <si>
+    <t>After each player move, an adjacent enemy deals one-round damage, retreats one cell away, and records its map position.</t>
+  </si>
+  <si>
+    <t>计算伤害时，敌人的防御力视为不低于对方攻击力-1。</t>
+  </si>
+  <si>
+    <t>战斗中计算伤害时，敌人将对方防御力视为0。</t>
+  </si>
+  <si>
+    <t>战斗中，敌人每回合基础伤害会按连击数倍计算。</t>
+  </si>
+  <si>
+    <t>敌人的攻击力视为不低于对方攻击力。</t>
+  </si>
+  <si>
+    <t>玩家每次移动后，若处于敌人的曼哈顿领域范围内，敌人造成一次单回合伤害。</t>
+  </si>
+  <si>
+    <t>玩家每次移动后，若被两个正对相邻的敌人夹在中间，二者各造成一次单回合伤害。</t>
+  </si>
+  <si>
+    <t>玩家每次移动后，相邻的敌人造成一次单回合伤害，向远离玩家方向后退一格，并记录地图坐标。</t>
+  </si>
+  <si>
+    <t>敌人在战败后会变身为另一敌人。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>The enemy will turn to another kind after this battle.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>GHOST_SOLDIER</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>GHOST_SOLDIER_DESC</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ghost Soldier</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>This is a ghost soldier.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>这是一个鬼战士。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>鬼战士</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1842,7 +1890,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -1941,13 +1989,13 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="B18" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="C18" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -2183,13 +2231,13 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>438</v>
+        <v>424</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>439</v>
+        <v>425</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>440</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -2200,7 +2248,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="43.1640625" customWidth="1"/>
@@ -2299,143 +2347,165 @@
       <c r="A9" t="s">
         <v>341</v>
       </c>
-      <c r="B9" t="s">
-        <v>342</v>
+      <c r="B9" s="4" t="s">
+        <v>446</v>
       </c>
       <c r="C9" t="s">
-        <v>343</v>
+        <v>453</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>342</v>
+      </c>
+      <c r="B10" t="s">
+        <v>343</v>
+      </c>
+      <c r="C10" t="s">
         <v>344</v>
-      </c>
-      <c r="B10" t="s">
-        <v>345</v>
-      </c>
-      <c r="C10" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B11" t="s">
-        <v>348</v>
-      </c>
-      <c r="C11" t="s">
-        <v>349</v>
+        <v>447</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B12" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="C12" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="B13" t="s">
-        <v>354</v>
+        <v>448</v>
       </c>
       <c r="C13" t="s">
-        <v>355</v>
+        <v>455</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="B14" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="C14" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="B15" t="s">
-        <v>360</v>
+        <v>449</v>
       </c>
       <c r="C15" t="s">
-        <v>361</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="B16" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="C16" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="B17" t="s">
-        <v>366</v>
+        <v>450</v>
       </c>
       <c r="C17" t="s">
-        <v>367</v>
+        <v>457</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
       <c r="B18" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="C18" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
       <c r="B19" t="s">
-        <v>372</v>
+        <v>451</v>
       </c>
       <c r="C19" t="s">
-        <v>373</v>
+        <v>458</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="B20" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="C20" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="B21" t="s">
-        <v>378</v>
+        <v>452</v>
       </c>
       <c r="C21" t="s">
-        <v>379</v>
+        <v>459</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -2466,24 +2536,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>380</v>
+        <v>366</v>
       </c>
       <c r="B2" t="s">
-        <v>381</v>
+        <v>367</v>
       </c>
       <c r="C2" t="s">
-        <v>382</v>
+        <v>368</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>383</v>
+        <v>369</v>
       </c>
       <c r="B3" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="C3" t="s">
-        <v>385</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -2515,35 +2585,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>392</v>
+        <v>378</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>390</v>
+        <v>376</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>391</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>420</v>
+        <v>406</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>423</v>
+        <v>409</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>422</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -2574,134 +2644,134 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>393</v>
+        <v>379</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>394</v>
+        <v>380</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>417</v>
+        <v>403</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>405</v>
+        <v>391</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>418</v>
+        <v>404</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>424</v>
+        <v>410</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>425</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>426</v>
+        <v>412</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>429</v>
+        <v>415</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>430</v>
+        <v>416</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>427</v>
+        <v>413</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>431</v>
+        <v>417</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>432</v>
+        <v>418</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>428</v>
+        <v>414</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>433</v>
+        <v>419</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>434</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -3195,68 +3265,68 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>435</v>
+        <v>421</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>444</v>
+        <v>430</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>441</v>
+        <v>427</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>447</v>
+        <v>433</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>451</v>
+        <v>437</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>436</v>
+        <v>422</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>445</v>
+        <v>431</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>442</v>
+        <v>428</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>448</v>
+        <v>434</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>454</v>
+        <v>440</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>453</v>
+        <v>439</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>437</v>
+        <v>423</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>446</v>
+        <v>432</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>443</v>
+        <v>429</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>449</v>
+        <v>435</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>455</v>
+        <v>441</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>452</v>
+        <v>438</v>
       </c>
     </row>
   </sheetData>
@@ -3267,7 +3337,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.58203125" customWidth="1"/>
@@ -3504,6 +3574,28 @@
       </c>
       <c r="C21" s="3" t="s">
         <v>277</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>466</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update antialiasinglevel configs and tilesets
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Other\Ludork\Sample\Data\Locale\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fengmingliu/Dev/Ludork/Sample/Data/Locale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B02A8BF-1E70-4343-B9E8-65FC89320410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E8AA3F-1D5D-D64C-BF06-843CDA960A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="940" yWindow="890" windowWidth="38420" windowHeight="19620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="2" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="471">
   <si>
     <t>ID</t>
   </si>
@@ -1511,13 +1511,22 @@
   <si>
     <t>鬼战士</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>antialiasinglevel</t>
+  </si>
+  <si>
+    <t>Antialiasing Level</t>
+  </si>
+  <si>
+    <t>抗锯齿等级</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1527,12 +1536,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="4"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1582,7 +1593,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1792,15 +1803,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C40"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.4140625" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="17.25" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1811,7 +1822,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1822,7 +1833,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1833,7 +1844,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1844,7 +1855,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1855,7 +1866,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1866,7 +1877,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1877,7 +1888,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1888,7 +1899,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" s="4" t="s">
         <v>375</v>
       </c>
@@ -1899,7 +1910,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1910,7 +1921,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1921,7 +1932,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1932,7 +1943,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1943,7 +1954,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -1954,7 +1965,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -1965,7 +1976,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>41</v>
       </c>
@@ -1976,7 +1987,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -1987,7 +1998,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>372</v>
       </c>
@@ -1998,7 +2009,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -2009,7 +2020,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>49</v>
       </c>
@@ -2020,7 +2031,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -2031,7 +2042,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>55</v>
       </c>
@@ -2042,7 +2053,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>58</v>
       </c>
@@ -2053,7 +2064,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>61</v>
       </c>
@@ -2064,179 +2075,190 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="25" spans="1:3">
+      <c r="A25" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>65</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
         <v>67</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>68</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
         <v>70</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>71</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
         <v>73</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>74</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
         <v>76</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>77</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
         <v>79</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>80</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
         <v>82</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>83</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
         <v>85</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>86</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C33" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
         <v>88</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>89</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
         <v>91</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>92</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C35" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
         <v>94</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>95</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C36" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
         <v>97</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>98</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C37" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
         <v>100</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>101</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C38" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
         <v>103</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>104</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
+    <row r="40" spans="1:3">
+      <c r="A40" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B40" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C40" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
+    <row r="41" spans="1:3">
+      <c r="A41" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B41" s="4" t="s">
         <v>425</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C41" s="4" t="s">
         <v>426</v>
       </c>
     </row>
@@ -2249,13 +2271,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="43.1640625" customWidth="1"/>
-    <col min="3" max="3" width="43.58203125" customWidth="1"/>
+    <col min="3" max="3" width="43.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2266,7 +2288,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -2277,7 +2299,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>325</v>
       </c>
@@ -2288,7 +2310,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>328</v>
       </c>
@@ -2299,7 +2321,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>330</v>
       </c>
@@ -2310,7 +2332,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>333</v>
       </c>
@@ -2321,7 +2343,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>335</v>
       </c>
@@ -2332,7 +2354,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>338</v>
       </c>
@@ -2343,7 +2365,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>341</v>
       </c>
@@ -2354,7 +2376,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>342</v>
       </c>
@@ -2365,7 +2387,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>345</v>
       </c>
@@ -2376,7 +2398,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>346</v>
       </c>
@@ -2387,7 +2409,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>349</v>
       </c>
@@ -2398,7 +2420,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>350</v>
       </c>
@@ -2409,7 +2431,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>353</v>
       </c>
@@ -2420,7 +2442,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>354</v>
       </c>
@@ -2431,7 +2453,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>357</v>
       </c>
@@ -2442,7 +2464,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>358</v>
       </c>
@@ -2453,7 +2475,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>361</v>
       </c>
@@ -2464,7 +2486,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>362</v>
       </c>
@@ -2475,7 +2497,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>365</v>
       </c>
@@ -2486,7 +2508,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22" s="4" t="s">
         <v>442</v>
       </c>
@@ -2497,7 +2519,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="A23" s="4" t="s">
         <v>445</v>
       </c>
@@ -2517,13 +2539,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="25.75" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2534,7 +2556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>366</v>
       </c>
@@ -2545,7 +2567,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>369</v>
       </c>
@@ -2565,14 +2587,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FA4E9DF-B4C0-496C-83E9-11467FE432C9}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.4140625" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.25" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2583,7 +2605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
         <v>378</v>
       </c>
@@ -2594,7 +2616,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
         <v>406</v>
       </c>
@@ -2605,7 +2627,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
         <v>407</v>
       </c>
@@ -2625,13 +2647,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18A9F10C-3E5E-41A2-9938-5DC7A61B6D47}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="34.58203125" customWidth="1"/>
-    <col min="3" max="3" width="34.5" customWidth="1"/>
+    <col min="2" max="3" width="34.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2642,7 +2663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
         <v>379</v>
       </c>
@@ -2653,7 +2674,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" s="4" t="s">
         <v>382</v>
       </c>
@@ -2664,7 +2685,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
         <v>399</v>
       </c>
@@ -2675,7 +2696,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" s="4" t="s">
         <v>400</v>
       </c>
@@ -2686,7 +2707,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" s="4" t="s">
         <v>401</v>
       </c>
@@ -2697,7 +2718,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
         <v>402</v>
       </c>
@@ -2708,7 +2729,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" s="4" t="s">
         <v>403</v>
       </c>
@@ -2719,7 +2740,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" s="4" t="s">
         <v>404</v>
       </c>
@@ -2730,7 +2751,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" s="4" t="s">
         <v>405</v>
       </c>
@@ -2741,7 +2762,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" s="4" t="s">
         <v>412</v>
       </c>
@@ -2752,7 +2773,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" s="4" t="s">
         <v>413</v>
       </c>
@@ -2763,7 +2784,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3">
       <c r="A13" s="4" t="s">
         <v>414</v>
       </c>
@@ -2783,9 +2804,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2796,7 +2817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2807,7 +2828,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2827,9 +2848,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2840,7 +2861,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
         <v>113</v>
       </c>
@@ -2851,7 +2872,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
         <v>116</v>
       </c>
@@ -2862,7 +2883,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>119</v>
       </c>
@@ -2873,7 +2894,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
         <v>121</v>
       </c>
@@ -2884,7 +2905,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
         <v>123</v>
       </c>
@@ -2895,7 +2916,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
         <v>125</v>
       </c>
@@ -2906,7 +2927,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
         <v>128</v>
       </c>
@@ -2917,7 +2938,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
         <v>131</v>
       </c>
@@ -2928,7 +2949,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
         <v>134</v>
       </c>
@@ -2939,7 +2960,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
         <v>137</v>
       </c>
@@ -2959,14 +2980,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.75" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2977,7 +2998,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>140</v>
       </c>
@@ -2988,7 +3009,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>143</v>
       </c>
@@ -2999,7 +3020,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>146</v>
       </c>
@@ -3010,7 +3031,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>149</v>
       </c>
@@ -3021,7 +3042,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>152</v>
       </c>
@@ -3032,7 +3053,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>155</v>
       </c>
@@ -3043,7 +3064,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>158</v>
       </c>
@@ -3054,7 +3075,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>161</v>
       </c>
@@ -3065,7 +3086,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>164</v>
       </c>
@@ -3076,7 +3097,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>167</v>
       </c>
@@ -3087,7 +3108,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>170</v>
       </c>
@@ -3098,7 +3119,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>173</v>
       </c>
@@ -3109,7 +3130,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>176</v>
       </c>
@@ -3120,7 +3141,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>179</v>
       </c>
@@ -3131,7 +3152,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>182</v>
       </c>
@@ -3142,7 +3163,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>185</v>
       </c>
@@ -3153,7 +3174,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>188</v>
       </c>
@@ -3164,7 +3185,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>191</v>
       </c>
@@ -3175,7 +3196,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>194</v>
       </c>
@@ -3186,7 +3207,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>197</v>
       </c>
@@ -3197,7 +3218,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>200</v>
       </c>
@@ -3208,7 +3229,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>203</v>
       </c>
@@ -3219,7 +3240,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>206</v>
       </c>
@@ -3230,7 +3251,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>209</v>
       </c>
@@ -3241,7 +3262,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>212</v>
       </c>
@@ -3252,7 +3273,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>215</v>
       </c>
@@ -3263,7 +3284,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3">
       <c r="A28" s="4" t="s">
         <v>421</v>
       </c>
@@ -3274,7 +3295,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3">
       <c r="A29" s="4" t="s">
         <v>433</v>
       </c>
@@ -3285,7 +3306,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3">
       <c r="A30" s="4" t="s">
         <v>422</v>
       </c>
@@ -3296,7 +3317,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3">
       <c r="A31" s="4" t="s">
         <v>434</v>
       </c>
@@ -3307,7 +3328,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3">
       <c r="A32" s="4" t="s">
         <v>423</v>
       </c>
@@ -3318,7 +3339,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3">
       <c r="A33" s="4" t="s">
         <v>435</v>
       </c>
@@ -3338,14 +3359,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.58203125" customWidth="1"/>
+    <col min="1" max="1" width="29.5" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="32.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3356,7 +3377,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>218</v>
       </c>
@@ -3367,7 +3388,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>221</v>
       </c>
@@ -3378,7 +3399,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>224</v>
       </c>
@@ -3389,7 +3410,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>227</v>
       </c>
@@ -3400,7 +3421,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>230</v>
       </c>
@@ -3411,7 +3432,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>233</v>
       </c>
@@ -3422,7 +3443,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>236</v>
       </c>
@@ -3433,7 +3454,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>239</v>
       </c>
@@ -3444,7 +3465,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>242</v>
       </c>
@@ -3455,7 +3476,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>245</v>
       </c>
@@ -3466,7 +3487,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>248</v>
       </c>
@@ -3477,7 +3498,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>251</v>
       </c>
@@ -3488,7 +3509,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3">
       <c r="A14" s="2" t="s">
         <v>254</v>
       </c>
@@ -3499,7 +3520,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3">
       <c r="A15" s="2" t="s">
         <v>257</v>
       </c>
@@ -3510,7 +3531,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
         <v>260</v>
       </c>
@@ -3521,7 +3542,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3">
       <c r="A17" s="2" t="s">
         <v>263</v>
       </c>
@@ -3532,7 +3553,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>266</v>
       </c>
@@ -3543,7 +3564,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19" s="2" t="s">
         <v>269</v>
       </c>
@@ -3554,7 +3575,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>272</v>
       </c>
@@ -3565,7 +3586,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3">
       <c r="A21" s="3" t="s">
         <v>275</v>
       </c>
@@ -3576,7 +3597,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22" s="4" t="s">
         <v>462</v>
       </c>
@@ -3587,7 +3608,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3">
       <c r="A23" s="4" t="s">
         <v>463</v>
       </c>
@@ -3607,13 +3628,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="52.9140625" customWidth="1"/>
+    <col min="2" max="2" width="52.83203125" customWidth="1"/>
     <col min="3" max="3" width="42.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3624,7 +3645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>278</v>
       </c>
@@ -3635,7 +3656,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>281</v>
       </c>
@@ -3646,7 +3667,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>284</v>
       </c>
@@ -3657,7 +3678,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>287</v>
       </c>
@@ -3677,13 +3698,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="35.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3694,7 +3715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>290</v>
       </c>
@@ -3705,7 +3726,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>293</v>
       </c>
@@ -3725,13 +3746,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="43.25" customWidth="1"/>
-    <col min="3" max="3" width="44.08203125" customWidth="1"/>
+    <col min="2" max="2" width="43.1640625" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3742,7 +3763,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>296</v>
       </c>
@@ -3753,7 +3774,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>299</v>
       </c>
@@ -3764,7 +3785,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>302</v>
       </c>
@@ -3775,7 +3796,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>305</v>
       </c>
@@ -3786,7 +3807,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>308</v>
       </c>
@@ -3806,14 +3827,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.08203125" customWidth="1"/>
-    <col min="3" max="3" width="17.25" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3824,7 +3845,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>311</v>
       </c>
@@ -3835,7 +3856,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>314</v>
       </c>
@@ -3846,7 +3867,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>317</v>
       </c>
@@ -3857,7 +3878,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>320</v>
       </c>

</xml_diff>

<commit_message>
Add an independent lighting render scale, overlay DropBox popups in Canvas, and tabbed Config quality presets.  This keeps lighting cheaper than the System canvas, stops expanded DropBoxes from resizing parent layout, and retargets HarmonyOS to API 22 free-window scale plus sectioned docs preview
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" r:id="Rf5f2439c2c6a494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Languages" sheetId="12" r:id="R31d6cf3603b1447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrs" sheetId="3" r:id="Rc9cb65dc915d48bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="Rfee6b8b610aa417b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="5" r:id="R04f2e8968b2a4f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="6" r:id="R0b82220b445c4e4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="7" r:id="R4c750b0eeefe4a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="8" r:id="Re2c048a7cba74a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="9" r:id="R30f8ba25fd8546fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="10" r:id="Refb195a68d734154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="11" r:id="R404a114adbc64d77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueNames" sheetId="13" r:id="R8ab02f9dde6d4ad9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueContents" sheetId="14" r:id="R87fe3329e03845ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" r:id="R7c6102095ac046a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Languages" sheetId="12" r:id="R6fd3ba9604ce46dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrs" sheetId="3" r:id="Rcb16155260ca416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="R08593f07489048da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="5" r:id="Ra38e1412645541fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="6" r:id="R82ae3d75aafe4b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="7" r:id="R7c8a05caf61f437e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="8" r:id="Rb73ecf821f834d99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="9" r:id="R7f29443a380e4d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="10" r:id="R57fb59fdebbe49aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="11" r:id="R10ede87ac49b4a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueNames" sheetId="13" r:id="R90c33be79393461e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueContents" sheetId="14" r:id="Rce66ef665e1d48a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2153,10 +2153,10 @@
         <x:v>maxrenderscale</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>Maximum Render Scale</x:v>
+        <x:v>Render Limit</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>最大渲染倍率</x:v>
+        <x:v>渲染上限</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2168,6 +2168,116 @@
       </x:c>
       <x:c r="C43" t="str">
         <x:v>不限</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>graphics</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>Graphics</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>画质</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>audio</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>Audio</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>音量</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>graphicspreset</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>Quality Preset</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>画质档位</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>lightingrenderscale</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>Lighting Resolution</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>光照分辨率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>low</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>低</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>medium</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>中</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>high</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>高</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>extrahigh</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>Extra High</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>超高</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>original</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>Original</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>原画</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>custom</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>Custom</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>自定义</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update tab view component
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" r:id="R7c6102095ac046a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Languages" sheetId="12" r:id="R6fd3ba9604ce46dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrs" sheetId="3" r:id="Rcb16155260ca416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="R08593f07489048da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="5" r:id="Ra38e1412645541fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="6" r:id="R82ae3d75aafe4b0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="7" r:id="R7c8a05caf61f437e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="8" r:id="Rb73ecf821f834d99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="9" r:id="R7f29443a380e4d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="10" r:id="R57fb59fdebbe49aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="11" r:id="R10ede87ac49b4a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueNames" sheetId="13" r:id="R90c33be79393461e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueContents" sheetId="14" r:id="Rce66ef665e1d48a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" r:id="R936406ca3ca44419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Languages" sheetId="12" r:id="Rb13e3c717c6a43ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrs" sheetId="3" r:id="R635c17cf092a4ae1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="R250cb1b3caee42e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="5" r:id="Re8421290e5f442c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="6" r:id="R41d10fce622c4250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="7" r:id="R0731ea360ed241ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="8" r:id="R5c2bf0bc8836409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="9" r:id="R63e35b6cb46d445d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="10" r:id="R8d4000e61aeb4aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="11" r:id="R2805da4dc25c4cd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueNames" sheetId="13" r:id="Rc1fe707b5fcb4790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueContents" sheetId="14" r:id="Reffa9329b2e84c09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2280,6 +2280,17 @@
         <x:v>自定义</x:v>
       </x:c>
     </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>other</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>Other</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>其他</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>